<commit_message>
docs(hop): them sheet Tong quan he thong Tien giam dinh, ra soat cau loi thoi
Sheet dau tien: he thong lam gi, quy mo du lieu/danh muc, ket qua kiem ky 01-15/10 (chan/canh bao/sach, T_BHTT),
theo co so/loai KCB/bang XML/don vi, top loi, chuyen bien sau nap lai, cai tien, viec can lam, muc luc.
Sua Trong tam D6/D10/D16/E16/D17/E17 va Ghi chu A3.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/hop/phan-loai-loi-tien-giam-dinh-theo-don-vi.xlsx
+++ b/docs/hop/phan-loai-loi-tien-giam-dinh-theo-don-vi.xlsx
@@ -3,20 +3,22 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="28800" windowHeight="12180" tabRatio="500" firstSheet="0" activeTab="4" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" windowWidth="28800" windowHeight="12180" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Tổng hợp" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Trọng tâm theo đơn vị" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Tài khoản thay CCHN" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Danh mục lỗi" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Đối chiếu FIXERROR" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Ghi chú" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Tổng quan hệ thống" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tổng hợp" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Trọng tâm theo đơn vị" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Tài khoản thay CCHN" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Danh mục lỗi" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Đối chiếu FIXERROR" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Ghi chú" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Danh mục lỗi'!$A$4:$P$222</definedName>
-    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Danh mục lỗi'!$4:$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Đối chiếu FIXERROR'!$A$4:$K$63</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Tổng quan hệ thống'!$A$1:$G$155</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Danh mục lỗi'!$A$4:$P$222</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Danh mục lỗi'!$4:$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Đối chiếu FIXERROR'!$A$4:$K$63</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -24,11 +26,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="#,##0;\-#,##0;&quot;&quot;"/>
+    <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="167" formatCode="+#,##0;-#,##0;0"/>
   </numFmts>
-  <fonts count="32">
+  <fonts count="38">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -253,8 +257,41 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="001F4E78"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill/>
     </fill>
@@ -453,8 +490,13 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="10">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -572,6 +614,64 @@
       </top>
       <bottom style="double">
         <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
       </bottom>
       <diagonal/>
     </border>
@@ -713,7 +813,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -750,6 +850,58 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="165" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="34" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="35" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="35" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="37" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="37" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="37" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="35" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="35" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="37" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="167" fontId="35" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1301,6 +1453,3137 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:G155"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="17" customWidth="1" min="6" max="6"/>
+    <col width="58" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="20" customHeight="1">
+      <c r="A1" s="20" t="inlineStr">
+        <is>
+          <t>BÁO CÁO TỔNG QUAN HỆ THỐNG TIỀN GIÁM ĐỊNH XML3176</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="21" t="inlineStr">
+        <is>
+          <t>Kỳ báo cáo: hồ sơ BHYT ra viện 01/10–15/10/2026 tại cơ sở 01929 và 37470 (dữ liệu nạp lại ngày 16/10/2026). Số liệu chốt ngày 16/10/2026 từ CSDL thật (truy vấn chỉ đọc); bộ kiểm commit 63e21fa8. Các ô tính từ sheet khác là công thức, tự cập nhật khi sheet nguồn thay đổi.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="A4" s="22" t="inlineStr">
+        <is>
+          <t>1. Hệ thống Tiền giám định làm gì</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="23" t="inlineStr">
+        <is>
+          <t>• Mục đích: kiểm tra hồ sơ XML theo Quyết định 3176/QĐ-BYT TRƯỚC khi gửi cổng giám định BHXH, phát hiện sai sót để sửa tại nguồn (HIS, PACS/LIS, danh mục, khoa/phòng), giảm hồ sơ bị BHXH từ chối hoặc xuất toán.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="30" customHeight="1">
+      <c r="A6" s="23" t="inlineStr">
+        <is>
+          <t>• Luồng xử lý: (1) Nạp XML từ HIS → (2) Kiểm tự động từng hồ sơ: 12 bảng XML và kiểm tổng thể toàn hồ sơ (XMLComplete) → (3) Có lỗi CHẶN GỬI: hồ sơ dừng, đơn vị sửa rồi nạp lại; chỉ có CẢNH BÁO: hồ sơ đi tiếp → (4) Xuất XML, ký số → (5) Gửi cổng giám định BHXH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="23" t="inlineStr">
+        <is>
+          <t>• Nguyên tắc: không tự sửa dữ liệu trên bản gửi cổng (khác hệ thống FIXERROR – xem sheet "Đối chiếu FIXERROR"); mỗi mã lỗi gán một đơn vị chủ trì và đơn vị phối hợp để giao việc (sheet "Danh mục lỗi").</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="22" t="inlineStr">
+        <is>
+          <t>2. Quy mô dữ liệu và danh mục</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>Chỉ tiêu</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>Giá trị</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+      <c r="D10" s="25" t="n"/>
+      <c r="E10" s="25" t="n"/>
+      <c r="F10" s="25" t="n"/>
+      <c r="G10" s="26" t="n"/>
+    </row>
+    <row r="11" ht="16.5" customHeight="1">
+      <c r="A11" s="27" t="inlineStr">
+        <is>
+          <t>Hồ sơ trong kỳ</t>
+        </is>
+      </c>
+      <c r="B11" s="28" t="n">
+        <v>23967</v>
+      </c>
+      <c r="C11" s="27" t="inlineStr">
+        <is>
+          <t>Cơ sở 01929: 18.845; cơ sở 37470: 5.122</t>
+        </is>
+      </c>
+      <c r="D11" s="29" t="n"/>
+      <c r="E11" s="29" t="n"/>
+      <c r="F11" s="29" t="n"/>
+      <c r="G11" s="29" t="n"/>
+    </row>
+    <row r="12" ht="16.5" customHeight="1">
+      <c r="A12" s="27" t="inlineStr">
+        <is>
+          <t>Dòng chi tiết được kiểm</t>
+        </is>
+      </c>
+      <c r="B12" s="28" t="n">
+        <v>3816571</v>
+      </c>
+      <c r="C12" s="27" t="inlineStr">
+        <is>
+          <t>Thuốc XML2: 560.375; DVKT/VTYT XML3: 955.173; cận lâm sàng XML4: 2.091.705; diễn biến XML5: 209.318</t>
+        </is>
+      </c>
+      <c r="D12" s="29" t="n"/>
+      <c r="E12" s="29" t="n"/>
+      <c r="F12" s="29" t="n"/>
+      <c r="G12" s="29" t="n"/>
+    </row>
+    <row r="13" ht="16.5" customHeight="1">
+      <c r="A13" s="27" t="inlineStr">
+        <is>
+          <t>Chi phí BHYT thanh toán (T_BHTT, tỷ đồng)</t>
+        </is>
+      </c>
+      <c r="B13" s="30" t="n">
+        <v>216.33</v>
+      </c>
+      <c r="C13" s="27" t="inlineStr">
+        <is>
+          <t>Tổng T_BHTT trên XML1 của các hồ sơ trong kỳ</t>
+        </is>
+      </c>
+      <c r="D13" s="29" t="n"/>
+      <c r="E13" s="29" t="n"/>
+      <c r="F13" s="29" t="n"/>
+      <c r="G13" s="29" t="n"/>
+    </row>
+    <row r="14" ht="16.5" customHeight="1">
+      <c r="A14" s="27" t="inlineStr">
+        <is>
+          <t>Mã lỗi trong danh mục</t>
+        </is>
+      </c>
+      <c r="B14" s="28" t="n">
+        <v>252</v>
+      </c>
+      <c r="C14" s="27" t="inlineStr">
+        <is>
+          <t>Đang kiểm 215 mã, trong đó 137 mã chặn gửi; còn lại đã tắt hoặc đã gộp vào mã mới</t>
+        </is>
+      </c>
+      <c r="D14" s="29" t="n"/>
+      <c r="E14" s="29" t="n"/>
+      <c r="F14" s="29" t="n"/>
+      <c r="G14" s="29" t="n"/>
+    </row>
+    <row r="15" ht="16.5" customHeight="1">
+      <c r="A15" s="27" t="inlineStr">
+        <is>
+          <t>Mã lỗi phát sinh trong kỳ</t>
+        </is>
+      </c>
+      <c r="B15" s="28">
+        <f>COUNTIF('Danh mục lỗi'!$G$5:$G$222,"&gt;0")</f>
+        <v/>
+      </c>
+      <c r="C15" s="27" t="inlineStr">
+        <is>
+          <t>Đếm từ sheet "Danh mục lỗi"</t>
+        </is>
+      </c>
+      <c r="D15" s="29" t="n"/>
+      <c r="E15" s="29" t="n"/>
+      <c r="F15" s="29" t="n"/>
+      <c r="G15" s="29" t="n"/>
+    </row>
+    <row r="16" ht="16.5" customHeight="1">
+      <c r="A16" s="27" t="inlineStr">
+        <is>
+          <t>Danh mục DVKT</t>
+        </is>
+      </c>
+      <c r="B16" s="28" t="n">
+        <v>24318</v>
+      </c>
+      <c r="C16" s="27" t="inlineStr">
+        <is>
+          <t>Cơ sở 01929: 8.595; cơ sở 37470: 15.723</t>
+        </is>
+      </c>
+      <c r="D16" s="29" t="n"/>
+      <c r="E16" s="29" t="n"/>
+      <c r="F16" s="29" t="n"/>
+      <c r="G16" s="29" t="n"/>
+    </row>
+    <row r="17" ht="16.5" customHeight="1">
+      <c r="A17" s="27" t="inlineStr">
+        <is>
+          <t>Danh mục thuốc</t>
+        </is>
+      </c>
+      <c r="B17" s="28" t="n">
+        <v>8689</v>
+      </c>
+      <c r="C17" s="27" t="inlineStr"/>
+      <c r="D17" s="29" t="n"/>
+      <c r="E17" s="29" t="n"/>
+      <c r="F17" s="29" t="n"/>
+      <c r="G17" s="29" t="n"/>
+    </row>
+    <row r="18" ht="16.5" customHeight="1">
+      <c r="A18" s="27" t="inlineStr">
+        <is>
+          <t>Danh mục VTYT</t>
+        </is>
+      </c>
+      <c r="B18" s="28" t="n">
+        <v>5243</v>
+      </c>
+      <c r="C18" s="27" t="inlineStr"/>
+      <c r="D18" s="29" t="n"/>
+      <c r="E18" s="29" t="n"/>
+      <c r="F18" s="29" t="n"/>
+      <c r="G18" s="29" t="n"/>
+    </row>
+    <row r="19" ht="16.5" customHeight="1">
+      <c r="A19" s="27" t="inlineStr">
+        <is>
+          <t>Danh mục nhân viên y tế (NVYT)</t>
+        </is>
+      </c>
+      <c r="B19" s="28" t="n">
+        <v>5089</v>
+      </c>
+      <c r="C19" s="27" t="inlineStr"/>
+      <c r="D19" s="29" t="n"/>
+      <c r="E19" s="29" t="n"/>
+      <c r="F19" s="29" t="n"/>
+      <c r="G19" s="29" t="n"/>
+    </row>
+    <row r="20" ht="16.5" customHeight="1">
+      <c r="A20" s="27" t="inlineStr">
+        <is>
+          <t>Danh mục trang thiết bị (mã máy)</t>
+        </is>
+      </c>
+      <c r="B20" s="28" t="n">
+        <v>8298</v>
+      </c>
+      <c r="C20" s="27" t="inlineStr"/>
+      <c r="D20" s="29" t="n"/>
+      <c r="E20" s="29" t="n"/>
+      <c r="F20" s="29" t="n"/>
+      <c r="G20" s="29" t="n"/>
+    </row>
+    <row r="21" ht="16.5" customHeight="1">
+      <c r="A21" s="27" t="inlineStr">
+        <is>
+          <t>DVKT bắt buộc có mã máy</t>
+        </is>
+      </c>
+      <c r="B21" s="28" t="n">
+        <v>3471</v>
+      </c>
+      <c r="C21" s="27" t="inlineStr">
+        <is>
+          <t>Căn cứ quy tắc thiếu mã máy từ 16/10/2026</t>
+        </is>
+      </c>
+      <c r="D21" s="29" t="n"/>
+      <c r="E21" s="29" t="n"/>
+      <c r="F21" s="29" t="n"/>
+      <c r="G21" s="29" t="n"/>
+    </row>
+    <row r="22" ht="16.5" customHeight="1">
+      <c r="A22" s="27" t="inlineStr">
+        <is>
+          <t>Cặp vật phẩm kèm DVKT</t>
+        </is>
+      </c>
+      <c r="B22" s="28" t="n">
+        <v>756</v>
+      </c>
+      <c r="C22" s="27" t="inlineStr">
+        <is>
+          <t>Thuốc/VTYT phải kèm đúng DVKT mẹ (quy tắc R1/R2)</t>
+        </is>
+      </c>
+      <c r="D22" s="29" t="n"/>
+      <c r="E22" s="29" t="n"/>
+      <c r="F22" s="29" t="n"/>
+      <c r="G22" s="29" t="n"/>
+    </row>
+    <row r="23" ht="16.5" customHeight="1">
+      <c r="A23" s="27" t="inlineStr">
+        <is>
+          <t>DVKT bắt buộc kèm vật phẩm</t>
+        </is>
+      </c>
+      <c r="B23" s="28" t="n">
+        <v>37</v>
+      </c>
+      <c r="C23" s="27" t="inlineStr">
+        <is>
+          <t>Quy tắc R3</t>
+        </is>
+      </c>
+      <c r="D23" s="29" t="n"/>
+      <c r="E23" s="29" t="n"/>
+      <c r="F23" s="29" t="n"/>
+      <c r="G23" s="29" t="n"/>
+    </row>
+    <row r="24" ht="16.5" customHeight="1">
+      <c r="A24" s="27" t="inlineStr">
+        <is>
+          <t>Danh mục cơ sở KCB</t>
+        </is>
+      </c>
+      <c r="B24" s="28" t="n">
+        <v>13843</v>
+      </c>
+      <c r="C24" s="27" t="inlineStr"/>
+      <c r="D24" s="29" t="n"/>
+      <c r="E24" s="29" t="n"/>
+      <c r="F24" s="29" t="n"/>
+      <c r="G24" s="29" t="n"/>
+    </row>
+    <row r="25" ht="16.5" customHeight="1">
+      <c r="A25" s="27" t="inlineStr">
+        <is>
+          <t>Danh mục ICD-10</t>
+        </is>
+      </c>
+      <c r="B25" s="28" t="n">
+        <v>17075</v>
+      </c>
+      <c r="C25" s="27" t="inlineStr"/>
+      <c r="D25" s="29" t="n"/>
+      <c r="E25" s="29" t="n"/>
+      <c r="F25" s="29" t="n"/>
+      <c r="G25" s="29" t="n"/>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="27" t="inlineStr">
+        <is>
+          <t>Tốc độ kiểm</t>
+        </is>
+      </c>
+      <c r="B26" s="27" t="inlineStr">
+        <is>
+          <t>≈ 0,26 giây/hồ sơ</t>
+        </is>
+      </c>
+      <c r="C26" s="27" t="inlineStr">
+        <is>
+          <t>Đo trên 200 hồ sơ mẫu ngày 15/10/2026; mỗi hồ sơ một lượt kiểm; sửa danh mục có hiệu lực ngay, không cần khởi động lại</t>
+        </is>
+      </c>
+      <c r="D26" s="29" t="n"/>
+      <c r="E26" s="29" t="n"/>
+      <c r="F26" s="29" t="n"/>
+      <c r="G26" s="29" t="n"/>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="22" t="inlineStr">
+        <is>
+          <t>3. Kết quả kiểm trong kỳ</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="24" t="inlineStr">
+        <is>
+          <t>Trạng thái hồ sơ</t>
+        </is>
+      </c>
+      <c r="B29" s="24" t="inlineStr">
+        <is>
+          <t>Số hồ sơ</t>
+        </is>
+      </c>
+      <c r="C29" s="24" t="inlineStr">
+        <is>
+          <t>% hồ sơ</t>
+        </is>
+      </c>
+      <c r="D29" s="24" t="inlineStr">
+        <is>
+          <t>T_BHTT (tỷ đồng)</t>
+        </is>
+      </c>
+      <c r="E29" s="24" t="inlineStr">
+        <is>
+          <t>% T_BHTT</t>
+        </is>
+      </c>
+      <c r="F29" s="24" t="inlineStr">
+        <is>
+          <t>Ý nghĩa</t>
+        </is>
+      </c>
+      <c r="G29" s="26" t="n"/>
+    </row>
+    <row r="30" ht="16.5" customHeight="1">
+      <c r="A30" s="31" t="inlineStr">
+        <is>
+          <t>Tổng hồ sơ</t>
+        </is>
+      </c>
+      <c r="B30" s="32" t="n">
+        <v>23967</v>
+      </c>
+      <c r="C30" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="34" t="n">
+        <v>216.33</v>
+      </c>
+      <c r="E30" s="33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="31" t="inlineStr"/>
+      <c r="G30" s="35" t="n"/>
+    </row>
+    <row r="31" ht="16.5" customHeight="1">
+      <c r="A31" s="27" t="inlineStr">
+        <is>
+          <t>Không có lỗi</t>
+        </is>
+      </c>
+      <c r="B31" s="28" t="n">
+        <v>1995</v>
+      </c>
+      <c r="C31" s="36">
+        <f>B31/$B$30</f>
+        <v/>
+      </c>
+      <c r="D31" s="30" t="n">
+        <v>3.44</v>
+      </c>
+      <c r="E31" s="36">
+        <f>D31/$D$30</f>
+        <v/>
+      </c>
+      <c r="F31" s="27" t="inlineStr">
+        <is>
+          <t>Đạt hoàn toàn</t>
+        </is>
+      </c>
+      <c r="G31" s="29" t="n"/>
+    </row>
+    <row r="32" ht="16.5" customHeight="1">
+      <c r="A32" s="27" t="inlineStr">
+        <is>
+          <t>Chỉ có cảnh báo</t>
+        </is>
+      </c>
+      <c r="B32" s="28" t="n">
+        <v>10432</v>
+      </c>
+      <c r="C32" s="36">
+        <f>B32/$B$30</f>
+        <v/>
+      </c>
+      <c r="D32" s="30" t="n">
+        <v>37.44</v>
+      </c>
+      <c r="E32" s="36">
+        <f>D32/$D$30</f>
+        <v/>
+      </c>
+      <c r="F32" s="27" t="inlineStr">
+        <is>
+          <t>Được xuất, ký, gửi nhưng có nguy cơ BHXH giảm trừ</t>
+        </is>
+      </c>
+      <c r="G32" s="29" t="n"/>
+    </row>
+    <row r="33" ht="16.5" customHeight="1">
+      <c r="A33" s="27" t="inlineStr">
+        <is>
+          <t>Bị chặn gửi (≥ 1 lỗi chặn)</t>
+        </is>
+      </c>
+      <c r="B33" s="28" t="n">
+        <v>11540</v>
+      </c>
+      <c r="C33" s="36">
+        <f>B33/$B$30</f>
+        <v/>
+      </c>
+      <c r="D33" s="30" t="n">
+        <v>175.45</v>
+      </c>
+      <c r="E33" s="36">
+        <f>D33/$D$30</f>
+        <v/>
+      </c>
+      <c r="F33" s="27" t="inlineStr">
+        <is>
+          <t>Không được xuất/ký/gửi đến khi sửa và nạp lại</t>
+        </is>
+      </c>
+      <c r="G33" s="29" t="n"/>
+    </row>
+    <row r="34" ht="16.5" customHeight="1">
+      <c r="A34" s="27" t="inlineStr">
+        <is>
+          <t>Đã xuất XML</t>
+        </is>
+      </c>
+      <c r="B34" s="28" t="n">
+        <v>12424</v>
+      </c>
+      <c r="C34" s="36">
+        <f>B34/$B$30</f>
+        <v/>
+      </c>
+      <c r="D34" s="27" t="inlineStr">
+        <is>
+          <t>Khớp số hồ sơ không bị chặn</t>
+        </is>
+      </c>
+      <c r="E34" s="29" t="n"/>
+      <c r="F34" s="29" t="n"/>
+      <c r="G34" s="29" t="n"/>
+    </row>
+    <row r="35" ht="16.5" customHeight="1">
+      <c r="A35" s="27" t="inlineStr">
+        <is>
+          <t>Đã ký số</t>
+        </is>
+      </c>
+      <c r="B35" s="28" t="n">
+        <v>12429</v>
+      </c>
+      <c r="C35" s="36">
+        <f>B35/$B$30</f>
+        <v/>
+      </c>
+      <c r="D35" s="27" t="inlineStr"/>
+      <c r="E35" s="29" t="n"/>
+      <c r="F35" s="29" t="n"/>
+      <c r="G35" s="29" t="n"/>
+    </row>
+    <row r="36" ht="16.5" customHeight="1">
+      <c r="A36" s="27" t="inlineStr">
+        <is>
+          <t>Đã gửi cổng qua Tiền giám định</t>
+        </is>
+      </c>
+      <c r="B36" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="C36" s="36">
+        <f>B36/$B$30</f>
+        <v/>
+      </c>
+      <c r="D36" s="27" t="inlineStr">
+        <is>
+          <t>Chưa gửi hồ sơ nào của kỳ này; lần gửi cổng gần nhất qua Tiền giám định là 29/09/2026</t>
+        </is>
+      </c>
+      <c r="E36" s="29" t="n"/>
+      <c r="F36" s="29" t="n"/>
+      <c r="G36" s="29" t="n"/>
+    </row>
+    <row r="38" ht="18" customHeight="1">
+      <c r="A38" s="22" t="inlineStr">
+        <is>
+          <t>4. Theo cơ sở KCB</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="30" customHeight="1">
+      <c r="A39" s="24" t="inlineStr">
+        <is>
+          <t>Cơ sở</t>
+        </is>
+      </c>
+      <c r="B39" s="24" t="inlineStr">
+        <is>
+          <t>Số hồ sơ</t>
+        </is>
+      </c>
+      <c r="C39" s="24" t="inlineStr">
+        <is>
+          <t>Bị chặn</t>
+        </is>
+      </c>
+      <c r="D39" s="24" t="inlineStr">
+        <is>
+          <t>% bị chặn</t>
+        </is>
+      </c>
+      <c r="E39" s="24" t="inlineStr">
+        <is>
+          <t>Không lỗi</t>
+        </is>
+      </c>
+      <c r="F39" s="24" t="inlineStr">
+        <is>
+          <t>T_BHTT (tỷ đồng)</t>
+        </is>
+      </c>
+      <c r="G39" s="24" t="inlineStr">
+        <is>
+          <t>T_BHTT hồ sơ bị chặn (tỷ đồng)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="16.5" customHeight="1">
+      <c r="A40" s="27" t="inlineStr">
+        <is>
+          <t>Cơ sở 01929</t>
+        </is>
+      </c>
+      <c r="B40" s="28" t="n">
+        <v>18845</v>
+      </c>
+      <c r="C40" s="28" t="n">
+        <v>9547</v>
+      </c>
+      <c r="D40" s="36">
+        <f>C40/B40</f>
+        <v/>
+      </c>
+      <c r="E40" s="28" t="n">
+        <v>1585</v>
+      </c>
+      <c r="F40" s="30" t="n">
+        <v>174.4</v>
+      </c>
+      <c r="G40" s="37" t="n">
+        <v>143.96</v>
+      </c>
+    </row>
+    <row r="41" ht="16.5" customHeight="1">
+      <c r="A41" s="27" t="inlineStr">
+        <is>
+          <t>Cơ sở 37470</t>
+        </is>
+      </c>
+      <c r="B41" s="28" t="n">
+        <v>5122</v>
+      </c>
+      <c r="C41" s="28" t="n">
+        <v>1993</v>
+      </c>
+      <c r="D41" s="36">
+        <f>C41/B41</f>
+        <v/>
+      </c>
+      <c r="E41" s="28" t="n">
+        <v>410</v>
+      </c>
+      <c r="F41" s="30" t="n">
+        <v>41.93</v>
+      </c>
+      <c r="G41" s="37" t="n">
+        <v>31.48</v>
+      </c>
+    </row>
+    <row r="42" ht="16.5" customHeight="1">
+      <c r="A42" s="31" t="inlineStr">
+        <is>
+          <t>Cộng</t>
+        </is>
+      </c>
+      <c r="B42" s="32">
+        <f>SUM(B40:B41)</f>
+        <v/>
+      </c>
+      <c r="C42" s="32">
+        <f>SUM(C40:C41)</f>
+        <v/>
+      </c>
+      <c r="D42" s="33">
+        <f>C42/B42</f>
+        <v/>
+      </c>
+      <c r="E42" s="32">
+        <f>SUM(E40:E41)</f>
+        <v/>
+      </c>
+      <c r="F42" s="34">
+        <f>SUM(F40:F41)</f>
+        <v/>
+      </c>
+      <c r="G42" s="38">
+        <f>SUM(G40:G41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44" ht="18" customHeight="1">
+      <c r="A44" s="22" t="inlineStr">
+        <is>
+          <t>5. Theo loại khám chữa bệnh (MA_LOAI_KCB)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="30" customHeight="1">
+      <c r="A45" s="24" t="inlineStr">
+        <is>
+          <t>Loại KCB</t>
+        </is>
+      </c>
+      <c r="B45" s="24" t="inlineStr">
+        <is>
+          <t>Số hồ sơ</t>
+        </is>
+      </c>
+      <c r="C45" s="24" t="inlineStr">
+        <is>
+          <t>Bị chặn</t>
+        </is>
+      </c>
+      <c r="D45" s="24" t="inlineStr">
+        <is>
+          <t>% bị chặn</t>
+        </is>
+      </c>
+      <c r="E45" s="24" t="inlineStr">
+        <is>
+          <t>Không lỗi</t>
+        </is>
+      </c>
+      <c r="F45" s="24" t="inlineStr">
+        <is>
+          <t>T_BHTT (tỷ đồng)</t>
+        </is>
+      </c>
+      <c r="G45" s="24" t="inlineStr">
+        <is>
+          <t>T_BHTT hồ sơ bị chặn (tỷ đồng)</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="16.5" customHeight="1">
+      <c r="A46" s="27" t="inlineStr">
+        <is>
+          <t>01 – Khám bệnh</t>
+        </is>
+      </c>
+      <c r="B46" s="28" t="n">
+        <v>10902</v>
+      </c>
+      <c r="C46" s="28" t="n">
+        <v>2578</v>
+      </c>
+      <c r="D46" s="36">
+        <f>C46/B46</f>
+        <v/>
+      </c>
+      <c r="E46" s="28" t="n">
+        <v>1957</v>
+      </c>
+      <c r="F46" s="30" t="n">
+        <v>27.02</v>
+      </c>
+      <c r="G46" s="37" t="n">
+        <v>7.7</v>
+      </c>
+    </row>
+    <row r="47" ht="16.5" customHeight="1">
+      <c r="A47" s="27" t="inlineStr">
+        <is>
+          <t>02 – Điều trị ngoại trú</t>
+        </is>
+      </c>
+      <c r="B47" s="28" t="n">
+        <v>1285</v>
+      </c>
+      <c r="C47" s="28" t="n">
+        <v>910</v>
+      </c>
+      <c r="D47" s="36">
+        <f>C47/B47</f>
+        <v/>
+      </c>
+      <c r="E47" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="F47" s="30" t="n">
+        <v>8</v>
+      </c>
+      <c r="G47" s="37" t="n">
+        <v>5.41</v>
+      </c>
+    </row>
+    <row r="48" ht="16.5" customHeight="1">
+      <c r="A48" s="27" t="inlineStr">
+        <is>
+          <t>03 – Điều trị nội trú</t>
+        </is>
+      </c>
+      <c r="B48" s="28" t="n">
+        <v>11271</v>
+      </c>
+      <c r="C48" s="28" t="n">
+        <v>7773</v>
+      </c>
+      <c r="D48" s="36">
+        <f>C48/B48</f>
+        <v/>
+      </c>
+      <c r="E48" s="28" t="n">
+        <v>19</v>
+      </c>
+      <c r="F48" s="30" t="n">
+        <v>178.6</v>
+      </c>
+      <c r="G48" s="37" t="n">
+        <v>160.04</v>
+      </c>
+    </row>
+    <row r="49" ht="16.5" customHeight="1">
+      <c r="A49" s="27" t="inlineStr">
+        <is>
+          <t>04 – Điều trị nội trú ban ngày</t>
+        </is>
+      </c>
+      <c r="B49" s="28" t="n">
+        <v>124</v>
+      </c>
+      <c r="C49" s="28" t="n">
+        <v>111</v>
+      </c>
+      <c r="D49" s="36">
+        <f>C49/B49</f>
+        <v/>
+      </c>
+      <c r="E49" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="30" t="n">
+        <v>2.24</v>
+      </c>
+      <c r="G49" s="37" t="n">
+        <v>2.11</v>
+      </c>
+    </row>
+    <row r="50" ht="16.5" customHeight="1">
+      <c r="A50" s="27" t="inlineStr">
+        <is>
+          <t>Mã 08</t>
+        </is>
+      </c>
+      <c r="B50" s="28" t="n">
+        <v>12</v>
+      </c>
+      <c r="C50" s="28" t="n">
+        <v>10</v>
+      </c>
+      <c r="D50" s="36">
+        <f>C50/B50</f>
+        <v/>
+      </c>
+      <c r="E50" s="28" t="n">
+        <v>0</v>
+      </c>
+      <c r="F50" s="30" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="G50" s="37" t="n">
+        <v>0.04</v>
+      </c>
+    </row>
+    <row r="51" ht="16.5" customHeight="1">
+      <c r="A51" s="27" t="inlineStr">
+        <is>
+          <t>09 – Điều trị nội trú dưới 4 giờ</t>
+        </is>
+      </c>
+      <c r="B51" s="28" t="n">
+        <v>373</v>
+      </c>
+      <c r="C51" s="28" t="n">
+        <v>158</v>
+      </c>
+      <c r="D51" s="36">
+        <f>C51/B51</f>
+        <v/>
+      </c>
+      <c r="E51" s="28" t="n">
+        <v>17</v>
+      </c>
+      <c r="F51" s="30" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="G51" s="37" t="n">
+        <v>0.16</v>
+      </c>
+    </row>
+    <row r="52" ht="16.5" customHeight="1">
+      <c r="A52" s="31" t="inlineStr">
+        <is>
+          <t>Cộng</t>
+        </is>
+      </c>
+      <c r="B52" s="32">
+        <f>SUM(B46:B51)</f>
+        <v/>
+      </c>
+      <c r="C52" s="32">
+        <f>SUM(C46:C51)</f>
+        <v/>
+      </c>
+      <c r="D52" s="33">
+        <f>C52/B52</f>
+        <v/>
+      </c>
+      <c r="E52" s="32">
+        <f>SUM(E46:E51)</f>
+        <v/>
+      </c>
+      <c r="F52" s="34">
+        <f>SUM(F46:F51)</f>
+        <v/>
+      </c>
+      <c r="G52" s="38">
+        <f>SUM(G46:G51)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54" ht="18" customHeight="1">
+      <c r="A54" s="22" t="inlineStr">
+        <is>
+          <t>6. Theo bảng XML</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="30" customHeight="1">
+      <c r="A55" s="24" t="inlineStr">
+        <is>
+          <t>Bảng</t>
+        </is>
+      </c>
+      <c r="B55" s="24" t="inlineStr">
+        <is>
+          <t>Mã lỗi đang kiểm</t>
+        </is>
+      </c>
+      <c r="C55" s="24" t="inlineStr">
+        <is>
+          <t>Trong đó chặn gửi</t>
+        </is>
+      </c>
+      <c r="D55" s="24" t="inlineStr">
+        <is>
+          <t>Hồ sơ có lỗi</t>
+        </is>
+      </c>
+      <c r="E55" s="24" t="inlineStr">
+        <is>
+          <t>% hồ sơ</t>
+        </is>
+      </c>
+      <c r="F55" s="24" t="inlineStr">
+        <is>
+          <t>Nội dung bảng</t>
+        </is>
+      </c>
+      <c r="G55" s="26" t="n"/>
+    </row>
+    <row r="56" ht="16.5" customHeight="1">
+      <c r="A56" s="27" t="inlineStr">
+        <is>
+          <t>XML1</t>
+        </is>
+      </c>
+      <c r="B56" s="28" t="n">
+        <v>48</v>
+      </c>
+      <c r="C56" s="28" t="n">
+        <v>39</v>
+      </c>
+      <c r="D56" s="28" t="n">
+        <v>945</v>
+      </c>
+      <c r="E56" s="36">
+        <f>D56/$B$30</f>
+        <v/>
+      </c>
+      <c r="F56" s="27" t="inlineStr">
+        <is>
+          <t>Thông tin tổng hợp hồ sơ, hành chính, chi phí</t>
+        </is>
+      </c>
+      <c r="G56" s="29" t="n"/>
+    </row>
+    <row r="57" ht="16.5" customHeight="1">
+      <c r="A57" s="27" t="inlineStr">
+        <is>
+          <t>XML2</t>
+        </is>
+      </c>
+      <c r="B57" s="28" t="n">
+        <v>25</v>
+      </c>
+      <c r="C57" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="D57" s="28" t="n">
+        <v>11240</v>
+      </c>
+      <c r="E57" s="36">
+        <f>D57/$B$30</f>
+        <v/>
+      </c>
+      <c r="F57" s="27" t="inlineStr">
+        <is>
+          <t>Thuốc</t>
+        </is>
+      </c>
+      <c r="G57" s="29" t="n"/>
+    </row>
+    <row r="58" ht="16.5" customHeight="1">
+      <c r="A58" s="27" t="inlineStr">
+        <is>
+          <t>XML3</t>
+        </is>
+      </c>
+      <c r="B58" s="28" t="n">
+        <v>56</v>
+      </c>
+      <c r="C58" s="28" t="n">
+        <v>24</v>
+      </c>
+      <c r="D58" s="28" t="n">
+        <v>20450</v>
+      </c>
+      <c r="E58" s="36">
+        <f>D58/$B$30</f>
+        <v/>
+      </c>
+      <c r="F58" s="27" t="inlineStr">
+        <is>
+          <t>Dịch vụ kỹ thuật và vật tư y tế</t>
+        </is>
+      </c>
+      <c r="G58" s="29" t="n"/>
+    </row>
+    <row r="59" ht="16.5" customHeight="1">
+      <c r="A59" s="27" t="inlineStr">
+        <is>
+          <t>XML4</t>
+        </is>
+      </c>
+      <c r="B59" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="C59" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="D59" s="28" t="n">
+        <v>18242</v>
+      </c>
+      <c r="E59" s="36">
+        <f>D59/$B$30</f>
+        <v/>
+      </c>
+      <c r="F59" s="27" t="inlineStr">
+        <is>
+          <t>Kết quả cận lâm sàng</t>
+        </is>
+      </c>
+      <c r="G59" s="29" t="n"/>
+    </row>
+    <row r="60" ht="16.5" customHeight="1">
+      <c r="A60" s="27" t="inlineStr">
+        <is>
+          <t>XML5</t>
+        </is>
+      </c>
+      <c r="B60" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="C60" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="D60" s="28" t="n">
+        <v>1584</v>
+      </c>
+      <c r="E60" s="36">
+        <f>D60/$B$30</f>
+        <v/>
+      </c>
+      <c r="F60" s="27" t="inlineStr">
+        <is>
+          <t>Diễn biến lâm sàng</t>
+        </is>
+      </c>
+      <c r="G60" s="29" t="n"/>
+    </row>
+    <row r="61" ht="16.5" customHeight="1">
+      <c r="A61" s="27" t="inlineStr">
+        <is>
+          <t>XML7</t>
+        </is>
+      </c>
+      <c r="B61" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="C61" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D61" s="28" t="n">
+        <v>643</v>
+      </c>
+      <c r="E61" s="36">
+        <f>D61/$B$30</f>
+        <v/>
+      </c>
+      <c r="F61" s="27" t="inlineStr">
+        <is>
+          <t>Giấy ra viện</t>
+        </is>
+      </c>
+      <c r="G61" s="29" t="n"/>
+    </row>
+    <row r="62" ht="16.5" customHeight="1">
+      <c r="A62" s="27" t="inlineStr">
+        <is>
+          <t>XML8</t>
+        </is>
+      </c>
+      <c r="B62" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="C62" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D62" s="28" t="n">
+        <v>7283</v>
+      </c>
+      <c r="E62" s="36">
+        <f>D62/$B$30</f>
+        <v/>
+      </c>
+      <c r="F62" s="27" t="inlineStr">
+        <is>
+          <t>Tóm tắt hồ sơ bệnh án</t>
+        </is>
+      </c>
+      <c r="G62" s="29" t="n"/>
+    </row>
+    <row r="63" ht="16.5" customHeight="1">
+      <c r="A63" s="27" t="inlineStr">
+        <is>
+          <t>XML9</t>
+        </is>
+      </c>
+      <c r="B63" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="C63" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="D63" s="28" t="n">
+        <v>10</v>
+      </c>
+      <c r="E63" s="36">
+        <f>D63/$B$30</f>
+        <v/>
+      </c>
+      <c r="F63" s="27" t="inlineStr">
+        <is>
+          <t>Giấy chứng sinh</t>
+        </is>
+      </c>
+      <c r="G63" s="29" t="n"/>
+    </row>
+    <row r="64" ht="16.5" customHeight="1">
+      <c r="A64" s="27" t="inlineStr">
+        <is>
+          <t>XML11</t>
+        </is>
+      </c>
+      <c r="B64" s="28" t="n">
+        <v>13</v>
+      </c>
+      <c r="C64" s="28" t="n">
+        <v>13</v>
+      </c>
+      <c r="D64" s="28" t="n">
+        <v>26</v>
+      </c>
+      <c r="E64" s="36">
+        <f>D64/$B$30</f>
+        <v/>
+      </c>
+      <c r="F64" s="27" t="inlineStr">
+        <is>
+          <t>Giấy chứng nhận nghỉ việc hưởng BHXH</t>
+        </is>
+      </c>
+      <c r="G64" s="29" t="n"/>
+    </row>
+    <row r="65" ht="16.5" customHeight="1">
+      <c r="A65" s="27" t="inlineStr">
+        <is>
+          <t>XML13</t>
+        </is>
+      </c>
+      <c r="B65" s="28" t="n">
+        <v>14</v>
+      </c>
+      <c r="C65" s="28" t="n">
+        <v>14</v>
+      </c>
+      <c r="D65" s="28" t="n">
+        <v>3</v>
+      </c>
+      <c r="E65" s="36">
+        <f>D65/$B$30</f>
+        <v/>
+      </c>
+      <c r="F65" s="27" t="inlineStr">
+        <is>
+          <t>Giấy chuyển tuyến</t>
+        </is>
+      </c>
+      <c r="G65" s="29" t="n"/>
+    </row>
+    <row r="66" ht="16.5" customHeight="1">
+      <c r="A66" s="27" t="inlineStr">
+        <is>
+          <t>XML14</t>
+        </is>
+      </c>
+      <c r="B66" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="C66" s="28" t="n">
+        <v>4</v>
+      </c>
+      <c r="D66" s="28" t="n">
+        <v>362</v>
+      </c>
+      <c r="E66" s="36">
+        <f>D66/$B$30</f>
+        <v/>
+      </c>
+      <c r="F66" s="27" t="inlineStr">
+        <is>
+          <t>Giấy hẹn khám lại</t>
+        </is>
+      </c>
+      <c r="G66" s="29" t="n"/>
+    </row>
+    <row r="67" ht="30" customHeight="1">
+      <c r="A67" s="27" t="inlineStr">
+        <is>
+          <t>XMLComplete</t>
+        </is>
+      </c>
+      <c r="B67" s="28" t="n">
+        <v>32</v>
+      </c>
+      <c r="C67" s="28" t="n">
+        <v>16</v>
+      </c>
+      <c r="D67" s="28" t="n">
+        <v>13232</v>
+      </c>
+      <c r="E67" s="36">
+        <f>D67/$B$30</f>
+        <v/>
+      </c>
+      <c r="F67" s="27" t="inlineStr">
+        <is>
+          <t>Kiểm tổng thể: đối chiếu chéo giữa các bảng, NVYT, ngày giường, mức hưởng, vật phẩm kèm DVKT</t>
+        </is>
+      </c>
+      <c r="G67" s="29" t="n"/>
+    </row>
+    <row r="69" ht="18" customHeight="1">
+      <c r="A69" s="22" t="inlineStr">
+        <is>
+          <t>7. Theo đơn vị chủ trì xử lý (tự lấy từ sheet "Tổng hợp")</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="30" customHeight="1">
+      <c r="A70" s="24" t="inlineStr">
+        <is>
+          <t>Đơn vị chủ trì</t>
+        </is>
+      </c>
+      <c r="B70" s="24" t="inlineStr">
+        <is>
+          <t>Số mã lỗi phát sinh</t>
+        </is>
+      </c>
+      <c r="C70" s="24" t="inlineStr">
+        <is>
+          <t>Trong đó chặn gửi</t>
+        </is>
+      </c>
+      <c r="D70" s="24" t="inlineStr">
+        <is>
+          <t>Lượt hồ sơ-lỗi</t>
+        </is>
+      </c>
+      <c r="E70" s="24" t="inlineStr">
+        <is>
+          <t>Lượt hồ sơ-lỗi chặn gửi</t>
+        </is>
+      </c>
+      <c r="F70" s="24" t="inlineStr">
+        <is>
+          <t>Mã lỗi lớn nhất</t>
+        </is>
+      </c>
+      <c r="G70" s="26" t="n"/>
+    </row>
+    <row r="71" ht="16.5" customHeight="1">
+      <c r="A71" s="27">
+        <f>'Tổng hợp'!A6</f>
+        <v/>
+      </c>
+      <c r="B71" s="28">
+        <f>'Tổng hợp'!B6</f>
+        <v/>
+      </c>
+      <c r="C71" s="28">
+        <f>'Tổng hợp'!C6</f>
+        <v/>
+      </c>
+      <c r="D71" s="28">
+        <f>'Tổng hợp'!D6</f>
+        <v/>
+      </c>
+      <c r="E71" s="28">
+        <f>'Tổng hợp'!E6</f>
+        <v/>
+      </c>
+      <c r="F71" s="27">
+        <f>IF('Tổng hợp'!F6="","",'Tổng hợp'!F6)</f>
+        <v/>
+      </c>
+      <c r="G71" s="29" t="n"/>
+    </row>
+    <row r="72" ht="16.5" customHeight="1">
+      <c r="A72" s="27">
+        <f>'Tổng hợp'!A7</f>
+        <v/>
+      </c>
+      <c r="B72" s="28">
+        <f>'Tổng hợp'!B7</f>
+        <v/>
+      </c>
+      <c r="C72" s="28">
+        <f>'Tổng hợp'!C7</f>
+        <v/>
+      </c>
+      <c r="D72" s="28">
+        <f>'Tổng hợp'!D7</f>
+        <v/>
+      </c>
+      <c r="E72" s="28">
+        <f>'Tổng hợp'!E7</f>
+        <v/>
+      </c>
+      <c r="F72" s="27">
+        <f>IF('Tổng hợp'!F7="","",'Tổng hợp'!F7)</f>
+        <v/>
+      </c>
+      <c r="G72" s="29" t="n"/>
+    </row>
+    <row r="73" ht="16.5" customHeight="1">
+      <c r="A73" s="27">
+        <f>'Tổng hợp'!A8</f>
+        <v/>
+      </c>
+      <c r="B73" s="28">
+        <f>'Tổng hợp'!B8</f>
+        <v/>
+      </c>
+      <c r="C73" s="28">
+        <f>'Tổng hợp'!C8</f>
+        <v/>
+      </c>
+      <c r="D73" s="28">
+        <f>'Tổng hợp'!D8</f>
+        <v/>
+      </c>
+      <c r="E73" s="28">
+        <f>'Tổng hợp'!E8</f>
+        <v/>
+      </c>
+      <c r="F73" s="27">
+        <f>IF('Tổng hợp'!F8="","",'Tổng hợp'!F8)</f>
+        <v/>
+      </c>
+      <c r="G73" s="29" t="n"/>
+    </row>
+    <row r="74" ht="16.5" customHeight="1">
+      <c r="A74" s="27">
+        <f>'Tổng hợp'!A9</f>
+        <v/>
+      </c>
+      <c r="B74" s="28">
+        <f>'Tổng hợp'!B9</f>
+        <v/>
+      </c>
+      <c r="C74" s="28">
+        <f>'Tổng hợp'!C9</f>
+        <v/>
+      </c>
+      <c r="D74" s="28">
+        <f>'Tổng hợp'!D9</f>
+        <v/>
+      </c>
+      <c r="E74" s="28">
+        <f>'Tổng hợp'!E9</f>
+        <v/>
+      </c>
+      <c r="F74" s="27">
+        <f>IF('Tổng hợp'!F9="","",'Tổng hợp'!F9)</f>
+        <v/>
+      </c>
+      <c r="G74" s="29" t="n"/>
+    </row>
+    <row r="75" ht="16.5" customHeight="1">
+      <c r="A75" s="27">
+        <f>'Tổng hợp'!A10</f>
+        <v/>
+      </c>
+      <c r="B75" s="28">
+        <f>'Tổng hợp'!B10</f>
+        <v/>
+      </c>
+      <c r="C75" s="28">
+        <f>'Tổng hợp'!C10</f>
+        <v/>
+      </c>
+      <c r="D75" s="28">
+        <f>'Tổng hợp'!D10</f>
+        <v/>
+      </c>
+      <c r="E75" s="28">
+        <f>'Tổng hợp'!E10</f>
+        <v/>
+      </c>
+      <c r="F75" s="27">
+        <f>IF('Tổng hợp'!F10="","",'Tổng hợp'!F10)</f>
+        <v/>
+      </c>
+      <c r="G75" s="29" t="n"/>
+    </row>
+    <row r="76" ht="16.5" customHeight="1">
+      <c r="A76" s="27">
+        <f>'Tổng hợp'!A11</f>
+        <v/>
+      </c>
+      <c r="B76" s="28">
+        <f>'Tổng hợp'!B11</f>
+        <v/>
+      </c>
+      <c r="C76" s="28">
+        <f>'Tổng hợp'!C11</f>
+        <v/>
+      </c>
+      <c r="D76" s="28">
+        <f>'Tổng hợp'!D11</f>
+        <v/>
+      </c>
+      <c r="E76" s="28">
+        <f>'Tổng hợp'!E11</f>
+        <v/>
+      </c>
+      <c r="F76" s="27">
+        <f>IF('Tổng hợp'!F11="","",'Tổng hợp'!F11)</f>
+        <v/>
+      </c>
+      <c r="G76" s="29" t="n"/>
+    </row>
+    <row r="77" ht="16.5" customHeight="1">
+      <c r="A77" s="27">
+        <f>'Tổng hợp'!A12</f>
+        <v/>
+      </c>
+      <c r="B77" s="28">
+        <f>'Tổng hợp'!B12</f>
+        <v/>
+      </c>
+      <c r="C77" s="28">
+        <f>'Tổng hợp'!C12</f>
+        <v/>
+      </c>
+      <c r="D77" s="28">
+        <f>'Tổng hợp'!D12</f>
+        <v/>
+      </c>
+      <c r="E77" s="28">
+        <f>'Tổng hợp'!E12</f>
+        <v/>
+      </c>
+      <c r="F77" s="27">
+        <f>IF('Tổng hợp'!F12="","",'Tổng hợp'!F12)</f>
+        <v/>
+      </c>
+      <c r="G77" s="29" t="n"/>
+    </row>
+    <row r="78" ht="16.5" customHeight="1">
+      <c r="A78" s="27">
+        <f>'Tổng hợp'!A13</f>
+        <v/>
+      </c>
+      <c r="B78" s="28">
+        <f>'Tổng hợp'!B13</f>
+        <v/>
+      </c>
+      <c r="C78" s="28">
+        <f>'Tổng hợp'!C13</f>
+        <v/>
+      </c>
+      <c r="D78" s="28">
+        <f>'Tổng hợp'!D13</f>
+        <v/>
+      </c>
+      <c r="E78" s="28">
+        <f>'Tổng hợp'!E13</f>
+        <v/>
+      </c>
+      <c r="F78" s="27">
+        <f>IF('Tổng hợp'!F13="","",'Tổng hợp'!F13)</f>
+        <v/>
+      </c>
+      <c r="G78" s="29" t="n"/>
+    </row>
+    <row r="79" ht="16.5" customHeight="1">
+      <c r="A79" s="27">
+        <f>'Tổng hợp'!A14</f>
+        <v/>
+      </c>
+      <c r="B79" s="28">
+        <f>'Tổng hợp'!B14</f>
+        <v/>
+      </c>
+      <c r="C79" s="28">
+        <f>'Tổng hợp'!C14</f>
+        <v/>
+      </c>
+      <c r="D79" s="28">
+        <f>'Tổng hợp'!D14</f>
+        <v/>
+      </c>
+      <c r="E79" s="28">
+        <f>'Tổng hợp'!E14</f>
+        <v/>
+      </c>
+      <c r="F79" s="27">
+        <f>IF('Tổng hợp'!F14="","",'Tổng hợp'!F14)</f>
+        <v/>
+      </c>
+      <c r="G79" s="29" t="n"/>
+    </row>
+    <row r="80" ht="16.5" customHeight="1">
+      <c r="A80" s="27">
+        <f>'Tổng hợp'!A15</f>
+        <v/>
+      </c>
+      <c r="B80" s="28">
+        <f>'Tổng hợp'!B15</f>
+        <v/>
+      </c>
+      <c r="C80" s="28">
+        <f>'Tổng hợp'!C15</f>
+        <v/>
+      </c>
+      <c r="D80" s="28">
+        <f>'Tổng hợp'!D15</f>
+        <v/>
+      </c>
+      <c r="E80" s="28">
+        <f>'Tổng hợp'!E15</f>
+        <v/>
+      </c>
+      <c r="F80" s="27">
+        <f>IF('Tổng hợp'!F15="","",'Tổng hợp'!F15)</f>
+        <v/>
+      </c>
+      <c r="G80" s="29" t="n"/>
+    </row>
+    <row r="81" ht="16.5" customHeight="1">
+      <c r="A81" s="31">
+        <f>'Tổng hợp'!A16</f>
+        <v/>
+      </c>
+      <c r="B81" s="32">
+        <f>'Tổng hợp'!B16</f>
+        <v/>
+      </c>
+      <c r="C81" s="32">
+        <f>'Tổng hợp'!C16</f>
+        <v/>
+      </c>
+      <c r="D81" s="32">
+        <f>'Tổng hợp'!D16</f>
+        <v/>
+      </c>
+      <c r="E81" s="32">
+        <f>'Tổng hợp'!E16</f>
+        <v/>
+      </c>
+      <c r="F81" s="31">
+        <f>IF('Tổng hợp'!F16="","",'Tổng hợp'!F16)</f>
+        <v/>
+      </c>
+      <c r="G81" s="35" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="21" t="inlineStr">
+        <is>
+          <t>"Lượt hồ sơ-lỗi" cộng số hồ sơ của từng mã, một hồ sơ nhiều lỗi được đếm nhiều lần – dùng để so sánh khối lượng việc giữa các đơn vị.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="18" customHeight="1">
+      <c r="A84" s="22" t="inlineStr">
+        <is>
+          <t>8. Mười lỗi CHẶN GỬI nhiều hồ sơ nhất</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="30" customHeight="1">
+      <c r="A85" s="24" t="inlineStr">
+        <is>
+          <t>Mã lỗi</t>
+        </is>
+      </c>
+      <c r="B85" s="24" t="inlineStr">
+        <is>
+          <t>Số hồ sơ</t>
+        </is>
+      </c>
+      <c r="C85" s="24" t="inlineStr">
+        <is>
+          <t>% hồ sơ</t>
+        </is>
+      </c>
+      <c r="D85" s="24" t="inlineStr">
+        <is>
+          <t>Đơn vị chủ trì</t>
+        </is>
+      </c>
+      <c r="E85" s="24" t="inlineStr">
+        <is>
+          <t>Tên lỗi</t>
+        </is>
+      </c>
+      <c r="F85" s="25" t="n"/>
+      <c r="G85" s="26" t="n"/>
+    </row>
+    <row r="86" ht="16.5" customHeight="1">
+      <c r="A86" s="27">
+        <f>'Danh mục lỗi'!B10</f>
+        <v/>
+      </c>
+      <c r="B86" s="28">
+        <f>'Danh mục lỗi'!G10</f>
+        <v/>
+      </c>
+      <c r="C86" s="36">
+        <f>'Danh mục lỗi'!G10/$B$30</f>
+        <v/>
+      </c>
+      <c r="D86" s="29">
+        <f>'Danh mục lỗi'!L10</f>
+        <v/>
+      </c>
+      <c r="E86" s="27">
+        <f>'Danh mục lỗi'!D10</f>
+        <v/>
+      </c>
+      <c r="F86" s="29" t="n"/>
+      <c r="G86" s="29" t="n"/>
+    </row>
+    <row r="87" ht="16.5" customHeight="1">
+      <c r="A87" s="27">
+        <f>'Danh mục lỗi'!B11</f>
+        <v/>
+      </c>
+      <c r="B87" s="28">
+        <f>'Danh mục lỗi'!G11</f>
+        <v/>
+      </c>
+      <c r="C87" s="36">
+        <f>'Danh mục lỗi'!G11/$B$30</f>
+        <v/>
+      </c>
+      <c r="D87" s="29">
+        <f>'Danh mục lỗi'!L11</f>
+        <v/>
+      </c>
+      <c r="E87" s="27">
+        <f>'Danh mục lỗi'!D11</f>
+        <v/>
+      </c>
+      <c r="F87" s="29" t="n"/>
+      <c r="G87" s="29" t="n"/>
+    </row>
+    <row r="88" ht="16.5" customHeight="1">
+      <c r="A88" s="27">
+        <f>'Danh mục lỗi'!B19</f>
+        <v/>
+      </c>
+      <c r="B88" s="28">
+        <f>'Danh mục lỗi'!G19</f>
+        <v/>
+      </c>
+      <c r="C88" s="36">
+        <f>'Danh mục lỗi'!G19/$B$30</f>
+        <v/>
+      </c>
+      <c r="D88" s="29">
+        <f>'Danh mục lỗi'!L19</f>
+        <v/>
+      </c>
+      <c r="E88" s="27">
+        <f>'Danh mục lỗi'!D19</f>
+        <v/>
+      </c>
+      <c r="F88" s="29" t="n"/>
+      <c r="G88" s="29" t="n"/>
+    </row>
+    <row r="89" ht="16.5" customHeight="1">
+      <c r="A89" s="27">
+        <f>'Danh mục lỗi'!B20</f>
+        <v/>
+      </c>
+      <c r="B89" s="28">
+        <f>'Danh mục lỗi'!G20</f>
+        <v/>
+      </c>
+      <c r="C89" s="36">
+        <f>'Danh mục lỗi'!G20/$B$30</f>
+        <v/>
+      </c>
+      <c r="D89" s="29">
+        <f>'Danh mục lỗi'!L20</f>
+        <v/>
+      </c>
+      <c r="E89" s="27">
+        <f>'Danh mục lỗi'!D20</f>
+        <v/>
+      </c>
+      <c r="F89" s="29" t="n"/>
+      <c r="G89" s="29" t="n"/>
+    </row>
+    <row r="90" ht="16.5" customHeight="1">
+      <c r="A90" s="27">
+        <f>'Danh mục lỗi'!B30</f>
+        <v/>
+      </c>
+      <c r="B90" s="28">
+        <f>'Danh mục lỗi'!G30</f>
+        <v/>
+      </c>
+      <c r="C90" s="36">
+        <f>'Danh mục lỗi'!G30/$B$30</f>
+        <v/>
+      </c>
+      <c r="D90" s="29">
+        <f>'Danh mục lỗi'!L30</f>
+        <v/>
+      </c>
+      <c r="E90" s="27">
+        <f>'Danh mục lỗi'!D30</f>
+        <v/>
+      </c>
+      <c r="F90" s="29" t="n"/>
+      <c r="G90" s="29" t="n"/>
+    </row>
+    <row r="91" ht="16.5" customHeight="1">
+      <c r="A91" s="27">
+        <f>'Danh mục lỗi'!B32</f>
+        <v/>
+      </c>
+      <c r="B91" s="28">
+        <f>'Danh mục lỗi'!G32</f>
+        <v/>
+      </c>
+      <c r="C91" s="36">
+        <f>'Danh mục lỗi'!G32/$B$30</f>
+        <v/>
+      </c>
+      <c r="D91" s="29">
+        <f>'Danh mục lỗi'!L32</f>
+        <v/>
+      </c>
+      <c r="E91" s="27">
+        <f>'Danh mục lỗi'!D32</f>
+        <v/>
+      </c>
+      <c r="F91" s="29" t="n"/>
+      <c r="G91" s="29" t="n"/>
+    </row>
+    <row r="92" ht="16.5" customHeight="1">
+      <c r="A92" s="27">
+        <f>'Danh mục lỗi'!B34</f>
+        <v/>
+      </c>
+      <c r="B92" s="28">
+        <f>'Danh mục lỗi'!G34</f>
+        <v/>
+      </c>
+      <c r="C92" s="36">
+        <f>'Danh mục lỗi'!G34/$B$30</f>
+        <v/>
+      </c>
+      <c r="D92" s="29">
+        <f>'Danh mục lỗi'!L34</f>
+        <v/>
+      </c>
+      <c r="E92" s="27">
+        <f>'Danh mục lỗi'!D34</f>
+        <v/>
+      </c>
+      <c r="F92" s="29" t="n"/>
+      <c r="G92" s="29" t="n"/>
+    </row>
+    <row r="93" ht="16.5" customHeight="1">
+      <c r="A93" s="27">
+        <f>'Danh mục lỗi'!B36</f>
+        <v/>
+      </c>
+      <c r="B93" s="28">
+        <f>'Danh mục lỗi'!G36</f>
+        <v/>
+      </c>
+      <c r="C93" s="36">
+        <f>'Danh mục lỗi'!G36/$B$30</f>
+        <v/>
+      </c>
+      <c r="D93" s="29">
+        <f>'Danh mục lỗi'!L36</f>
+        <v/>
+      </c>
+      <c r="E93" s="27">
+        <f>'Danh mục lỗi'!D36</f>
+        <v/>
+      </c>
+      <c r="F93" s="29" t="n"/>
+      <c r="G93" s="29" t="n"/>
+    </row>
+    <row r="94" ht="16.5" customHeight="1">
+      <c r="A94" s="27">
+        <f>'Danh mục lỗi'!B37</f>
+        <v/>
+      </c>
+      <c r="B94" s="28">
+        <f>'Danh mục lỗi'!G37</f>
+        <v/>
+      </c>
+      <c r="C94" s="36">
+        <f>'Danh mục lỗi'!G37/$B$30</f>
+        <v/>
+      </c>
+      <c r="D94" s="29">
+        <f>'Danh mục lỗi'!L37</f>
+        <v/>
+      </c>
+      <c r="E94" s="27">
+        <f>'Danh mục lỗi'!D37</f>
+        <v/>
+      </c>
+      <c r="F94" s="29" t="n"/>
+      <c r="G94" s="29" t="n"/>
+    </row>
+    <row r="95" ht="16.5" customHeight="1">
+      <c r="A95" s="27">
+        <f>'Danh mục lỗi'!B39</f>
+        <v/>
+      </c>
+      <c r="B95" s="28">
+        <f>'Danh mục lỗi'!G39</f>
+        <v/>
+      </c>
+      <c r="C95" s="36">
+        <f>'Danh mục lỗi'!G39/$B$30</f>
+        <v/>
+      </c>
+      <c r="D95" s="29">
+        <f>'Danh mục lỗi'!L39</f>
+        <v/>
+      </c>
+      <c r="E95" s="27">
+        <f>'Danh mục lỗi'!D39</f>
+        <v/>
+      </c>
+      <c r="F95" s="29" t="n"/>
+      <c r="G95" s="29" t="n"/>
+    </row>
+    <row r="97" ht="18" customHeight="1">
+      <c r="A97" s="22" t="inlineStr">
+        <is>
+          <t>9. Mười lỗi CẢNH BÁO nhiều hồ sơ nhất</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="30" customHeight="1">
+      <c r="A98" s="24" t="inlineStr">
+        <is>
+          <t>Mã lỗi</t>
+        </is>
+      </c>
+      <c r="B98" s="24" t="inlineStr">
+        <is>
+          <t>Số hồ sơ</t>
+        </is>
+      </c>
+      <c r="C98" s="24" t="inlineStr">
+        <is>
+          <t>% hồ sơ</t>
+        </is>
+      </c>
+      <c r="D98" s="24" t="inlineStr">
+        <is>
+          <t>Đơn vị chủ trì</t>
+        </is>
+      </c>
+      <c r="E98" s="24" t="inlineStr">
+        <is>
+          <t>Tên lỗi</t>
+        </is>
+      </c>
+      <c r="F98" s="25" t="n"/>
+      <c r="G98" s="26" t="n"/>
+    </row>
+    <row r="99" ht="16.5" customHeight="1">
+      <c r="A99" s="27">
+        <f>'Danh mục lỗi'!B5</f>
+        <v/>
+      </c>
+      <c r="B99" s="28">
+        <f>'Danh mục lỗi'!G5</f>
+        <v/>
+      </c>
+      <c r="C99" s="36">
+        <f>'Danh mục lỗi'!G5/$B$30</f>
+        <v/>
+      </c>
+      <c r="D99" s="29">
+        <f>'Danh mục lỗi'!L5</f>
+        <v/>
+      </c>
+      <c r="E99" s="27">
+        <f>'Danh mục lỗi'!D5</f>
+        <v/>
+      </c>
+      <c r="F99" s="29" t="n"/>
+      <c r="G99" s="29" t="n"/>
+    </row>
+    <row r="100" ht="16.5" customHeight="1">
+      <c r="A100" s="27">
+        <f>'Danh mục lỗi'!B6</f>
+        <v/>
+      </c>
+      <c r="B100" s="28">
+        <f>'Danh mục lỗi'!G6</f>
+        <v/>
+      </c>
+      <c r="C100" s="36">
+        <f>'Danh mục lỗi'!G6/$B$30</f>
+        <v/>
+      </c>
+      <c r="D100" s="29">
+        <f>'Danh mục lỗi'!L6</f>
+        <v/>
+      </c>
+      <c r="E100" s="27">
+        <f>'Danh mục lỗi'!D6</f>
+        <v/>
+      </c>
+      <c r="F100" s="29" t="n"/>
+      <c r="G100" s="29" t="n"/>
+    </row>
+    <row r="101" ht="16.5" customHeight="1">
+      <c r="A101" s="27">
+        <f>'Danh mục lỗi'!B7</f>
+        <v/>
+      </c>
+      <c r="B101" s="28">
+        <f>'Danh mục lỗi'!G7</f>
+        <v/>
+      </c>
+      <c r="C101" s="36">
+        <f>'Danh mục lỗi'!G7/$B$30</f>
+        <v/>
+      </c>
+      <c r="D101" s="29">
+        <f>'Danh mục lỗi'!L7</f>
+        <v/>
+      </c>
+      <c r="E101" s="27">
+        <f>'Danh mục lỗi'!D7</f>
+        <v/>
+      </c>
+      <c r="F101" s="29" t="n"/>
+      <c r="G101" s="29" t="n"/>
+    </row>
+    <row r="102" ht="16.5" customHeight="1">
+      <c r="A102" s="27">
+        <f>'Danh mục lỗi'!B8</f>
+        <v/>
+      </c>
+      <c r="B102" s="28">
+        <f>'Danh mục lỗi'!G8</f>
+        <v/>
+      </c>
+      <c r="C102" s="36">
+        <f>'Danh mục lỗi'!G8/$B$30</f>
+        <v/>
+      </c>
+      <c r="D102" s="29">
+        <f>'Danh mục lỗi'!L8</f>
+        <v/>
+      </c>
+      <c r="E102" s="27">
+        <f>'Danh mục lỗi'!D8</f>
+        <v/>
+      </c>
+      <c r="F102" s="29" t="n"/>
+      <c r="G102" s="29" t="n"/>
+    </row>
+    <row r="103" ht="16.5" customHeight="1">
+      <c r="A103" s="27">
+        <f>'Danh mục lỗi'!B9</f>
+        <v/>
+      </c>
+      <c r="B103" s="28">
+        <f>'Danh mục lỗi'!G9</f>
+        <v/>
+      </c>
+      <c r="C103" s="36">
+        <f>'Danh mục lỗi'!G9/$B$30</f>
+        <v/>
+      </c>
+      <c r="D103" s="29">
+        <f>'Danh mục lỗi'!L9</f>
+        <v/>
+      </c>
+      <c r="E103" s="27">
+        <f>'Danh mục lỗi'!D9</f>
+        <v/>
+      </c>
+      <c r="F103" s="29" t="n"/>
+      <c r="G103" s="29" t="n"/>
+    </row>
+    <row r="104" ht="16.5" customHeight="1">
+      <c r="A104" s="27">
+        <f>'Danh mục lỗi'!B12</f>
+        <v/>
+      </c>
+      <c r="B104" s="28">
+        <f>'Danh mục lỗi'!G12</f>
+        <v/>
+      </c>
+      <c r="C104" s="36">
+        <f>'Danh mục lỗi'!G12/$B$30</f>
+        <v/>
+      </c>
+      <c r="D104" s="29">
+        <f>'Danh mục lỗi'!L12</f>
+        <v/>
+      </c>
+      <c r="E104" s="27">
+        <f>'Danh mục lỗi'!D12</f>
+        <v/>
+      </c>
+      <c r="F104" s="29" t="n"/>
+      <c r="G104" s="29" t="n"/>
+    </row>
+    <row r="105" ht="16.5" customHeight="1">
+      <c r="A105" s="27">
+        <f>'Danh mục lỗi'!B13</f>
+        <v/>
+      </c>
+      <c r="B105" s="28">
+        <f>'Danh mục lỗi'!G13</f>
+        <v/>
+      </c>
+      <c r="C105" s="36">
+        <f>'Danh mục lỗi'!G13/$B$30</f>
+        <v/>
+      </c>
+      <c r="D105" s="29">
+        <f>'Danh mục lỗi'!L13</f>
+        <v/>
+      </c>
+      <c r="E105" s="27">
+        <f>'Danh mục lỗi'!D13</f>
+        <v/>
+      </c>
+      <c r="F105" s="29" t="n"/>
+      <c r="G105" s="29" t="n"/>
+    </row>
+    <row r="106" ht="16.5" customHeight="1">
+      <c r="A106" s="27">
+        <f>'Danh mục lỗi'!B14</f>
+        <v/>
+      </c>
+      <c r="B106" s="28">
+        <f>'Danh mục lỗi'!G14</f>
+        <v/>
+      </c>
+      <c r="C106" s="36">
+        <f>'Danh mục lỗi'!G14/$B$30</f>
+        <v/>
+      </c>
+      <c r="D106" s="29">
+        <f>'Danh mục lỗi'!L14</f>
+        <v/>
+      </c>
+      <c r="E106" s="27">
+        <f>'Danh mục lỗi'!D14</f>
+        <v/>
+      </c>
+      <c r="F106" s="29" t="n"/>
+      <c r="G106" s="29" t="n"/>
+    </row>
+    <row r="107" ht="16.5" customHeight="1">
+      <c r="A107" s="27">
+        <f>'Danh mục lỗi'!B15</f>
+        <v/>
+      </c>
+      <c r="B107" s="28">
+        <f>'Danh mục lỗi'!G15</f>
+        <v/>
+      </c>
+      <c r="C107" s="36">
+        <f>'Danh mục lỗi'!G15/$B$30</f>
+        <v/>
+      </c>
+      <c r="D107" s="29">
+        <f>'Danh mục lỗi'!L15</f>
+        <v/>
+      </c>
+      <c r="E107" s="27">
+        <f>'Danh mục lỗi'!D15</f>
+        <v/>
+      </c>
+      <c r="F107" s="29" t="n"/>
+      <c r="G107" s="29" t="n"/>
+    </row>
+    <row r="108" ht="16.5" customHeight="1">
+      <c r="A108" s="27">
+        <f>'Danh mục lỗi'!B16</f>
+        <v/>
+      </c>
+      <c r="B108" s="28">
+        <f>'Danh mục lỗi'!G16</f>
+        <v/>
+      </c>
+      <c r="C108" s="36">
+        <f>'Danh mục lỗi'!G16/$B$30</f>
+        <v/>
+      </c>
+      <c r="D108" s="29">
+        <f>'Danh mục lỗi'!L16</f>
+        <v/>
+      </c>
+      <c r="E108" s="27">
+        <f>'Danh mục lỗi'!D16</f>
+        <v/>
+      </c>
+      <c r="F108" s="29" t="n"/>
+      <c r="G108" s="29" t="n"/>
+    </row>
+    <row r="110" ht="18" customHeight="1">
+      <c r="A110" s="22" t="inlineStr">
+        <is>
+          <t>10. Chuyển biến sau khi sửa và nạp lại (cùng 23.254 hồ sơ có trong cả hai lần kiểm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="30" customHeight="1">
+      <c r="A111" s="24" t="inlineStr">
+        <is>
+          <t>Chỉ tiêu</t>
+        </is>
+      </c>
+      <c r="B111" s="24" t="inlineStr">
+        <is>
+          <t>Trước (kiểm sáng 16/10)</t>
+        </is>
+      </c>
+      <c r="C111" s="24" t="inlineStr">
+        <is>
+          <t>Sau (nạp lại 16/10)</t>
+        </is>
+      </c>
+      <c r="D111" s="24" t="inlineStr">
+        <is>
+          <t>Thay đổi</t>
+        </is>
+      </c>
+      <c r="E111" s="24" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+      <c r="F111" s="25" t="n"/>
+      <c r="G111" s="26" t="n"/>
+    </row>
+    <row r="112" ht="16.5" customHeight="1">
+      <c r="A112" s="27" t="inlineStr">
+        <is>
+          <t>Hồ sơ bị chặn gửi</t>
+        </is>
+      </c>
+      <c r="B112" s="28" t="n">
+        <v>11447</v>
+      </c>
+      <c r="C112" s="28" t="n">
+        <v>11087</v>
+      </c>
+      <c r="D112" s="39">
+        <f>C112-B112</f>
+        <v/>
+      </c>
+      <c r="E112" s="27" t="inlineStr">
+        <is>
+          <t>Hồ sơ đã sửa nguồn và nạp lại</t>
+        </is>
+      </c>
+      <c r="F112" s="29" t="n"/>
+      <c r="G112" s="29" t="n"/>
+    </row>
+    <row r="113" ht="16.5" customHeight="1">
+      <c r="A113" s="27" t="inlineStr">
+        <is>
+          <t>Hồ sơ không lỗi</t>
+        </is>
+      </c>
+      <c r="B113" s="28" t="n">
+        <v>1936</v>
+      </c>
+      <c r="C113" s="28" t="n">
+        <v>1981</v>
+      </c>
+      <c r="D113" s="39">
+        <f>C113-B113</f>
+        <v/>
+      </c>
+      <c r="E113" s="27" t="inlineStr"/>
+      <c r="F113" s="29" t="n"/>
+      <c r="G113" s="29" t="n"/>
+    </row>
+    <row r="114" ht="16.5" customHeight="1">
+      <c r="A114" s="27" t="inlineStr">
+        <is>
+          <t>XML4_INFO_ERROR_NGAY_KQ</t>
+        </is>
+      </c>
+      <c r="B114" s="28">
+        <f>INDEX('Danh mục lỗi'!$P$5:$P$222,MATCH("XML4_INFO_ERROR_NGAY_KQ",'Danh mục lỗi'!$B$5:$B$222,0))</f>
+        <v/>
+      </c>
+      <c r="C114" s="28">
+        <f>INDEX('Danh mục lỗi'!$G$5:$G$222,MATCH("XML4_INFO_ERROR_NGAY_KQ",'Danh mục lỗi'!$B$5:$B$222,0))</f>
+        <v/>
+      </c>
+      <c r="D114" s="39">
+        <f>C114-B114</f>
+        <v/>
+      </c>
+      <c r="E114" s="27" t="inlineStr">
+        <is>
+          <t>Giảm rõ</t>
+        </is>
+      </c>
+      <c r="F114" s="29" t="n"/>
+      <c r="G114" s="29" t="n"/>
+    </row>
+    <row r="115" ht="16.5" customHeight="1">
+      <c r="A115" s="27" t="inlineStr">
+        <is>
+          <t>XMLComplete_NVYT_THIEU</t>
+        </is>
+      </c>
+      <c r="B115" s="28">
+        <f>INDEX('Danh mục lỗi'!$P$5:$P$222,MATCH("XMLComplete_NVYT_THIEU",'Danh mục lỗi'!$B$5:$B$222,0))</f>
+        <v/>
+      </c>
+      <c r="C115" s="28">
+        <f>INDEX('Danh mục lỗi'!$G$5:$G$222,MATCH("XMLComplete_NVYT_THIEU",'Danh mục lỗi'!$B$5:$B$222,0))</f>
+        <v/>
+      </c>
+      <c r="D115" s="39">
+        <f>C115-B115</f>
+        <v/>
+      </c>
+      <c r="E115" s="27" t="inlineStr">
+        <is>
+          <t>Giảm</t>
+        </is>
+      </c>
+      <c r="F115" s="29" t="n"/>
+      <c r="G115" s="29" t="n"/>
+    </row>
+    <row r="116" ht="16.5" customHeight="1">
+      <c r="A116" s="27" t="inlineStr">
+        <is>
+          <t>XMLComplete_NVYT_SAI_DINH_DANG</t>
+        </is>
+      </c>
+      <c r="B116" s="28">
+        <f>INDEX('Danh mục lỗi'!$P$5:$P$222,MATCH("XMLComplete_NVYT_SAI_DINH_DANG",'Danh mục lỗi'!$B$5:$B$222,0))</f>
+        <v/>
+      </c>
+      <c r="C116" s="28">
+        <f>INDEX('Danh mục lỗi'!$G$5:$G$222,MATCH("XMLComplete_NVYT_SAI_DINH_DANG",'Danh mục lỗi'!$B$5:$B$222,0))</f>
+        <v/>
+      </c>
+      <c r="D116" s="39">
+        <f>C116-B116</f>
+        <v/>
+      </c>
+      <c r="E116" s="27" t="inlineStr">
+        <is>
+          <t>Giảm</t>
+        </is>
+      </c>
+      <c r="F116" s="29" t="n"/>
+      <c r="G116" s="29" t="n"/>
+    </row>
+    <row r="117" ht="16.5" customHeight="1">
+      <c r="A117" s="27" t="inlineStr">
+        <is>
+          <t>XML3_MA_DICH_VU_TB_CO_DON_GIA</t>
+        </is>
+      </c>
+      <c r="B117" s="28">
+        <f>INDEX('Danh mục lỗi'!$P$5:$P$222,MATCH("XML3_MA_DICH_VU_TB_CO_DON_GIA",'Danh mục lỗi'!$B$5:$B$222,0))</f>
+        <v/>
+      </c>
+      <c r="C117" s="28">
+        <f>INDEX('Danh mục lỗi'!$G$5:$G$222,MATCH("XML3_MA_DICH_VU_TB_CO_DON_GIA",'Danh mục lỗi'!$B$5:$B$222,0))</f>
+        <v/>
+      </c>
+      <c r="D117" s="39">
+        <f>C117-B117</f>
+        <v/>
+      </c>
+      <c r="E117" s="27" t="inlineStr">
+        <is>
+          <t>Hết lỗi</t>
+        </is>
+      </c>
+      <c r="F117" s="29" t="n"/>
+      <c r="G117" s="29" t="n"/>
+    </row>
+    <row r="118" ht="16.5" customHeight="1">
+      <c r="A118" s="27" t="inlineStr">
+        <is>
+          <t>XML3_INVALID_NGAY_KQ</t>
+        </is>
+      </c>
+      <c r="B118" s="28">
+        <f>INDEX('Danh mục lỗi'!$P$5:$P$222,MATCH("XML3_INVALID_NGAY_KQ",'Danh mục lỗi'!$B$5:$B$222,0))</f>
+        <v/>
+      </c>
+      <c r="C118" s="28">
+        <f>INDEX('Danh mục lỗi'!$G$5:$G$222,MATCH("XML3_INVALID_NGAY_KQ",'Danh mục lỗi'!$B$5:$B$222,0))</f>
+        <v/>
+      </c>
+      <c r="D118" s="39">
+        <f>C118-B118</f>
+        <v/>
+      </c>
+      <c r="E118" s="27" t="inlineStr">
+        <is>
+          <t>TĂNG gần gấp đôi – cần rà dữ liệu ngày kết quả trong lần xuất mới</t>
+        </is>
+      </c>
+      <c r="F118" s="29" t="n"/>
+      <c r="G118" s="29" t="n"/>
+    </row>
+    <row r="119" ht="26" customHeight="1">
+      <c r="A119" s="21" t="inlineStr">
+        <is>
+          <t>Dòng theo mã lỗi lấy từ sheet "Danh mục lỗi": cột "Trước" là cột P (chỉ gồm hồ sơ có trong lần kiểm sáng), cột "Sau" gồm cả 713 hồ sơ mới nạp lần đầu nên có thể nhích lên do thêm hồ sơ.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="18" customHeight="1">
+      <c r="A121" s="22" t="inlineStr">
+        <is>
+          <t>11. Cải tiến hệ thống trong kỳ</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="30" customHeight="1">
+      <c r="A122" s="24" t="inlineStr">
+        <is>
+          <t>Ngày</t>
+        </is>
+      </c>
+      <c r="B122" s="24" t="inlineStr">
+        <is>
+          <t>Nội dung</t>
+        </is>
+      </c>
+      <c r="C122" s="25" t="n"/>
+      <c r="D122" s="25" t="n"/>
+      <c r="E122" s="25" t="n"/>
+      <c r="F122" s="26" t="n"/>
+      <c r="G122" s="24" t="inlineStr">
+        <is>
+          <t>Tác dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="43.5" customHeight="1">
+      <c r="A123" s="27" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="B123" s="27" t="inlineStr">
+        <is>
+          <t>Sửa luật kiểm hàm lượng và thông tin thầu thuốc</t>
+        </is>
+      </c>
+      <c r="C123" s="29" t="n"/>
+      <c r="D123" s="29" t="n"/>
+      <c r="E123" s="29" t="n"/>
+      <c r="F123" s="29" t="n"/>
+      <c r="G123" s="27" t="inlineStr">
+        <is>
+          <t>Hết báo nhầm hàm lượng thành sai thầu – nguyên nhân của 85% chênh lệch khi đối chiếu giảm trừ với cổng ngày 12/10</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="30" customHeight="1">
+      <c r="A124" s="27" t="inlineStr">
+        <is>
+          <t>13/10/2026</t>
+        </is>
+      </c>
+      <c r="B124" s="27" t="inlineStr">
+        <is>
+          <t>Chứng từ điện tử: chặn ký/gửi khi thiếu số CCCD hoặc mã thẻ sai độ dài; màn quản trị vật phẩm kèm DVKT</t>
+        </is>
+      </c>
+      <c r="C124" s="29" t="n"/>
+      <c r="D124" s="29" t="n"/>
+      <c r="E124" s="29" t="n"/>
+      <c r="F124" s="29" t="n"/>
+      <c r="G124" s="27" t="inlineStr">
+        <is>
+          <t>Chặn sớm hồ sơ chắc chắn bị cổng từ chối</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="30" customHeight="1">
+      <c r="A125" s="27" t="inlineStr">
+        <is>
+          <t>14/10/2026</t>
+        </is>
+      </c>
+      <c r="B125" s="27" t="inlineStr">
+        <is>
+          <t>Đối chiếu mã DVKT có hậu tố _XX; quy tắc R1–R3 thuốc/VTYT kèm DVKT mẹ</t>
+        </is>
+      </c>
+      <c r="C125" s="29" t="n"/>
+      <c r="D125" s="29" t="n"/>
+      <c r="E125" s="29" t="n"/>
+      <c r="F125" s="29" t="n"/>
+      <c r="G125" s="27" t="inlineStr">
+        <is>
+          <t>Bỏ báo oan mã DVKT; phát hiện vật phẩm khai lệch DVKT</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="43.5" customHeight="1">
+      <c r="A126" s="27" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="B126" s="27" t="inlineStr">
+        <is>
+          <t>Gộp 34 mã lỗi NVYT thành 3 mã; gộp mã/tên chỉ số trống; lỗi chồng giờ PTTT và thời gian thực hiện dài bất thường; bỏ 16 chỗ báo trùng giữa quy tắc cũ và mới</t>
+        </is>
+      </c>
+      <c r="C126" s="29" t="n"/>
+      <c r="D126" s="29" t="n"/>
+      <c r="E126" s="29" t="n"/>
+      <c r="F126" s="29" t="n"/>
+      <c r="G126" s="27" t="inlineStr">
+        <is>
+          <t>Danh sách lỗi gọn, mỗi sai sót báo một lần, dễ giao việc</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="30" customHeight="1">
+      <c r="A127" s="27" t="inlineStr">
+        <is>
+          <t>15/10/2026</t>
+        </is>
+      </c>
+      <c r="B127" s="27" t="inlineStr">
+        <is>
+          <t>Tăng tốc kiểm: bộ đệm danh mục, chỉ mục CSDL, một lượt kiểm mỗi hồ sơ</t>
+        </is>
+      </c>
+      <c r="C127" s="29" t="n"/>
+      <c r="D127" s="29" t="n"/>
+      <c r="E127" s="29" t="n"/>
+      <c r="F127" s="29" t="n"/>
+      <c r="G127" s="27" t="inlineStr">
+        <is>
+          <t>309 → 256 ms/hồ sơ; truy vấn kiểm tổng thể giảm ~70%</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="30" customHeight="1">
+      <c r="A128" s="27" t="inlineStr">
+        <is>
+          <t>16/10/2026</t>
+        </is>
+      </c>
+      <c r="B128" s="27" t="inlineStr">
+        <is>
+          <t>Thiếu mã máy căn cứ danh mục DVKT bắt buộc có mã máy (thay lọc theo nhóm 1/2/3)</t>
+        </is>
+      </c>
+      <c r="C128" s="29" t="n"/>
+      <c r="D128" s="29" t="n"/>
+      <c r="E128" s="29" t="n"/>
+      <c r="F128" s="29" t="n"/>
+      <c r="G128" s="27" t="inlineStr">
+        <is>
+          <t>Kiểm đúng phạm vi BHXH yêu cầu; số hồ sơ thiếu mã máy tăng</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="18" customHeight="1">
+      <c r="A130" s="22" t="inlineStr">
+        <is>
+          <t>12. Việc cần làm theo đơn vị (tự lấy từ sheet "Trọng tâm theo đơn vị")</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="30" customHeight="1">
+      <c r="A131" s="24" t="inlineStr">
+        <is>
+          <t>Đơn vị</t>
+        </is>
+      </c>
+      <c r="B131" s="24" t="inlineStr">
+        <is>
+          <t>Vấn đề / số hồ sơ</t>
+        </is>
+      </c>
+      <c r="C131" s="25" t="n"/>
+      <c r="D131" s="25" t="n"/>
+      <c r="E131" s="25" t="n"/>
+      <c r="F131" s="26" t="n"/>
+      <c r="G131" s="24" t="inlineStr">
+        <is>
+          <t>Việc cần làm</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="30" customHeight="1">
+      <c r="A132" s="27">
+        <f>'Trọng tâm theo đơn vị'!B5</f>
+        <v/>
+      </c>
+      <c r="B132" s="29">
+        <f>'Trọng tâm theo đơn vị'!E5</f>
+        <v/>
+      </c>
+      <c r="C132" s="29" t="n"/>
+      <c r="D132" s="29" t="n"/>
+      <c r="E132" s="29" t="n"/>
+      <c r="F132" s="29" t="n"/>
+      <c r="G132" s="27">
+        <f>'Trọng tâm theo đơn vị'!F5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="133" ht="30" customHeight="1">
+      <c r="A133" s="27">
+        <f>'Trọng tâm theo đơn vị'!B6</f>
+        <v/>
+      </c>
+      <c r="B133" s="29">
+        <f>'Trọng tâm theo đơn vị'!E6</f>
+        <v/>
+      </c>
+      <c r="C133" s="29" t="n"/>
+      <c r="D133" s="29" t="n"/>
+      <c r="E133" s="29" t="n"/>
+      <c r="F133" s="29" t="n"/>
+      <c r="G133" s="27">
+        <f>'Trọng tâm theo đơn vị'!F6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="134" ht="30" customHeight="1">
+      <c r="A134" s="27">
+        <f>'Trọng tâm theo đơn vị'!B7</f>
+        <v/>
+      </c>
+      <c r="B134" s="29">
+        <f>'Trọng tâm theo đơn vị'!E7</f>
+        <v/>
+      </c>
+      <c r="C134" s="29" t="n"/>
+      <c r="D134" s="29" t="n"/>
+      <c r="E134" s="29" t="n"/>
+      <c r="F134" s="29" t="n"/>
+      <c r="G134" s="27">
+        <f>'Trọng tâm theo đơn vị'!F7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="135" ht="30" customHeight="1">
+      <c r="A135" s="27">
+        <f>'Trọng tâm theo đơn vị'!B8</f>
+        <v/>
+      </c>
+      <c r="B135" s="29">
+        <f>'Trọng tâm theo đơn vị'!E8</f>
+        <v/>
+      </c>
+      <c r="C135" s="29" t="n"/>
+      <c r="D135" s="29" t="n"/>
+      <c r="E135" s="29" t="n"/>
+      <c r="F135" s="29" t="n"/>
+      <c r="G135" s="27">
+        <f>'Trọng tâm theo đơn vị'!F8</f>
+        <v/>
+      </c>
+    </row>
+    <row r="136" ht="30" customHeight="1">
+      <c r="A136" s="27">
+        <f>'Trọng tâm theo đơn vị'!B9</f>
+        <v/>
+      </c>
+      <c r="B136" s="29">
+        <f>'Trọng tâm theo đơn vị'!E9</f>
+        <v/>
+      </c>
+      <c r="C136" s="29" t="n"/>
+      <c r="D136" s="29" t="n"/>
+      <c r="E136" s="29" t="n"/>
+      <c r="F136" s="29" t="n"/>
+      <c r="G136" s="27">
+        <f>'Trọng tâm theo đơn vị'!F9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="137" ht="30" customHeight="1">
+      <c r="A137" s="27">
+        <f>'Trọng tâm theo đơn vị'!B10</f>
+        <v/>
+      </c>
+      <c r="B137" s="29">
+        <f>'Trọng tâm theo đơn vị'!E10</f>
+        <v/>
+      </c>
+      <c r="C137" s="29" t="n"/>
+      <c r="D137" s="29" t="n"/>
+      <c r="E137" s="29" t="n"/>
+      <c r="F137" s="29" t="n"/>
+      <c r="G137" s="27">
+        <f>'Trọng tâm theo đơn vị'!F10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="138" ht="30" customHeight="1">
+      <c r="A138" s="27">
+        <f>'Trọng tâm theo đơn vị'!B11</f>
+        <v/>
+      </c>
+      <c r="B138" s="29">
+        <f>'Trọng tâm theo đơn vị'!E11</f>
+        <v/>
+      </c>
+      <c r="C138" s="29" t="n"/>
+      <c r="D138" s="29" t="n"/>
+      <c r="E138" s="29" t="n"/>
+      <c r="F138" s="29" t="n"/>
+      <c r="G138" s="27">
+        <f>'Trọng tâm theo đơn vị'!F11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="139" ht="30" customHeight="1">
+      <c r="A139" s="27">
+        <f>'Trọng tâm theo đơn vị'!B12</f>
+        <v/>
+      </c>
+      <c r="B139" s="29">
+        <f>'Trọng tâm theo đơn vị'!E12</f>
+        <v/>
+      </c>
+      <c r="C139" s="29" t="n"/>
+      <c r="D139" s="29" t="n"/>
+      <c r="E139" s="29" t="n"/>
+      <c r="F139" s="29" t="n"/>
+      <c r="G139" s="27">
+        <f>'Trọng tâm theo đơn vị'!F12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="140" ht="30" customHeight="1">
+      <c r="A140" s="27">
+        <f>'Trọng tâm theo đơn vị'!B13</f>
+        <v/>
+      </c>
+      <c r="B140" s="29">
+        <f>'Trọng tâm theo đơn vị'!E13</f>
+        <v/>
+      </c>
+      <c r="C140" s="29" t="n"/>
+      <c r="D140" s="29" t="n"/>
+      <c r="E140" s="29" t="n"/>
+      <c r="F140" s="29" t="n"/>
+      <c r="G140" s="27">
+        <f>'Trọng tâm theo đơn vị'!F13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="141" ht="30" customHeight="1">
+      <c r="A141" s="27">
+        <f>'Trọng tâm theo đơn vị'!B14</f>
+        <v/>
+      </c>
+      <c r="B141" s="29">
+        <f>'Trọng tâm theo đơn vị'!E14</f>
+        <v/>
+      </c>
+      <c r="C141" s="29" t="n"/>
+      <c r="D141" s="29" t="n"/>
+      <c r="E141" s="29" t="n"/>
+      <c r="F141" s="29" t="n"/>
+      <c r="G141" s="27">
+        <f>'Trọng tâm theo đơn vị'!F14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="142" ht="30" customHeight="1">
+      <c r="A142" s="27">
+        <f>'Trọng tâm theo đơn vị'!B15</f>
+        <v/>
+      </c>
+      <c r="B142" s="29">
+        <f>'Trọng tâm theo đơn vị'!E15</f>
+        <v/>
+      </c>
+      <c r="C142" s="29" t="n"/>
+      <c r="D142" s="29" t="n"/>
+      <c r="E142" s="29" t="n"/>
+      <c r="F142" s="29" t="n"/>
+      <c r="G142" s="27">
+        <f>'Trọng tâm theo đơn vị'!F15</f>
+        <v/>
+      </c>
+    </row>
+    <row r="143" ht="30" customHeight="1">
+      <c r="A143" s="27">
+        <f>'Trọng tâm theo đơn vị'!B16</f>
+        <v/>
+      </c>
+      <c r="B143" s="29">
+        <f>'Trọng tâm theo đơn vị'!E16</f>
+        <v/>
+      </c>
+      <c r="C143" s="29" t="n"/>
+      <c r="D143" s="29" t="n"/>
+      <c r="E143" s="29" t="n"/>
+      <c r="F143" s="29" t="n"/>
+      <c r="G143" s="27">
+        <f>'Trọng tâm theo đơn vị'!F16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="144" ht="30" customHeight="1">
+      <c r="A144" s="27">
+        <f>'Trọng tâm theo đơn vị'!B17</f>
+        <v/>
+      </c>
+      <c r="B144" s="29">
+        <f>'Trọng tâm theo đơn vị'!E17</f>
+        <v/>
+      </c>
+      <c r="C144" s="29" t="n"/>
+      <c r="D144" s="29" t="n"/>
+      <c r="E144" s="29" t="n"/>
+      <c r="F144" s="29" t="n"/>
+      <c r="G144" s="27">
+        <f>'Trọng tâm theo đơn vị'!F17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="145" ht="30" customHeight="1">
+      <c r="A145" s="27">
+        <f>'Trọng tâm theo đơn vị'!B18</f>
+        <v/>
+      </c>
+      <c r="B145" s="29">
+        <f>'Trọng tâm theo đơn vị'!E18</f>
+        <v/>
+      </c>
+      <c r="C145" s="29" t="n"/>
+      <c r="D145" s="29" t="n"/>
+      <c r="E145" s="29" t="n"/>
+      <c r="F145" s="29" t="n"/>
+      <c r="G145" s="27">
+        <f>'Trọng tâm theo đơn vị'!F18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="147" ht="18" customHeight="1">
+      <c r="A147" s="22" t="inlineStr">
+        <is>
+          <t>13. Các sheet trong tệp</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="30" customHeight="1">
+      <c r="A148" s="24" t="inlineStr">
+        <is>
+          <t>Sheet</t>
+        </is>
+      </c>
+      <c r="B148" s="24" t="inlineStr">
+        <is>
+          <t>Nội dung</t>
+        </is>
+      </c>
+      <c r="C148" s="25" t="n"/>
+      <c r="D148" s="25" t="n"/>
+      <c r="E148" s="25" t="n"/>
+      <c r="F148" s="26" t="n"/>
+      <c r="G148" s="24" t="inlineStr">
+        <is>
+          <t>Dùng khi</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="30" customHeight="1">
+      <c r="A149" s="27" t="inlineStr">
+        <is>
+          <t>Tổng quan hệ thống</t>
+        </is>
+      </c>
+      <c r="B149" s="27" t="inlineStr">
+        <is>
+          <t>Sheet này: hệ thống, quy mô, kết quả, chuyển biến, việc cần làm</t>
+        </is>
+      </c>
+      <c r="C149" s="29" t="n"/>
+      <c r="D149" s="29" t="n"/>
+      <c r="E149" s="29" t="n"/>
+      <c r="F149" s="29" t="n"/>
+      <c r="G149" s="27" t="inlineStr">
+        <is>
+          <t>Báo cáo lãnh đạo</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="30" customHeight="1">
+      <c r="A150" s="27" t="inlineStr">
+        <is>
+          <t>Tổng hợp</t>
+        </is>
+      </c>
+      <c r="B150" s="27" t="inlineStr">
+        <is>
+          <t>Số mã lỗi và lượt hồ sơ-lỗi theo đơn vị chủ trì và theo nhóm nghiệp vụ/kỹ thuật</t>
+        </is>
+      </c>
+      <c r="C150" s="29" t="n"/>
+      <c r="D150" s="29" t="n"/>
+      <c r="E150" s="29" t="n"/>
+      <c r="F150" s="29" t="n"/>
+      <c r="G150" s="27" t="inlineStr">
+        <is>
+          <t>So sánh khối lượng việc giữa các đơn vị</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="30" customHeight="1">
+      <c r="A151" s="27" t="inlineStr">
+        <is>
+          <t>Trọng tâm theo đơn vị</t>
+        </is>
+      </c>
+      <c r="B151" s="27" t="inlineStr">
+        <is>
+          <t>Vấn đề chính, số hồ sơ và việc cần làm của từng đơn vị</t>
+        </is>
+      </c>
+      <c r="C151" s="29" t="n"/>
+      <c r="D151" s="29" t="n"/>
+      <c r="E151" s="29" t="n"/>
+      <c r="F151" s="29" t="n"/>
+      <c r="G151" s="27" t="inlineStr">
+        <is>
+          <t>Giao việc trong cuộc họp</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="30" customHeight="1">
+      <c r="A152" s="27" t="inlineStr">
+        <is>
+          <t>Tài khoản thay CCHN</t>
+        </is>
+      </c>
+      <c r="B152" s="27" t="inlineStr">
+        <is>
+          <t>Tài khoản máy/tên đăng nhập/số định danh bị gửi thay mã CCHN</t>
+        </is>
+      </c>
+      <c r="C152" s="29" t="n"/>
+      <c r="D152" s="29" t="n"/>
+      <c r="E152" s="29" t="n"/>
+      <c r="F152" s="29" t="n"/>
+      <c r="G152" s="27" t="inlineStr">
+        <is>
+          <t>Làm việc với CNTT và hãng PACS/LIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="30" customHeight="1">
+      <c r="A153" s="27" t="inlineStr">
+        <is>
+          <t>Danh mục lỗi</t>
+        </is>
+      </c>
+      <c r="B153" s="27" t="inlineStr">
+        <is>
+          <t>Toàn bộ mã lỗi: chặn gửi, số hồ sơ, ví dụ thực tế, đơn vị chủ trì/phối hợp, hướng xử lý</t>
+        </is>
+      </c>
+      <c r="C153" s="29" t="n"/>
+      <c r="D153" s="29" t="n"/>
+      <c r="E153" s="29" t="n"/>
+      <c r="F153" s="29" t="n"/>
+      <c r="G153" s="27" t="inlineStr">
+        <is>
+          <t>Tra cứu một mã lỗi cụ thể</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="30" customHeight="1">
+      <c r="A154" s="27" t="inlineStr">
+        <is>
+          <t>Đối chiếu FIXERROR</t>
+        </is>
+      </c>
+      <c r="B154" s="27" t="inlineStr">
+        <is>
+          <t>Quy tắc tự sửa của hệ thống khác ↔ mã lỗi Tiền giám định tương ứng; cột Còn dùng/Ghi chú do team tool sửa XML cập nhật</t>
+        </is>
+      </c>
+      <c r="C154" s="29" t="n"/>
+      <c r="D154" s="29" t="n"/>
+      <c r="E154" s="29" t="n"/>
+      <c r="F154" s="29" t="n"/>
+      <c r="G154" s="27" t="inlineStr">
+        <is>
+          <t>Rà soát việc tự sửa dữ liệu trên bản gửi</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="30" customHeight="1">
+      <c r="A155" s="27" t="inlineStr">
+        <is>
+          <t>Ghi chú</t>
+        </is>
+      </c>
+      <c r="B155" s="27" t="inlineStr">
+        <is>
+          <t>Nguồn số liệu, cách đọc và quy ước phân loại</t>
+        </is>
+      </c>
+      <c r="C155" s="29" t="n"/>
+      <c r="D155" s="29" t="n"/>
+      <c r="E155" s="29" t="n"/>
+      <c r="F155" s="29" t="n"/>
+      <c r="G155" s="27" t="inlineStr">
+        <is>
+          <t>Khi cần giải thích số liệu</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="116">
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="E118:G118"/>
+    <mergeCell ref="B122:F122"/>
+    <mergeCell ref="C14:G14"/>
+    <mergeCell ref="B131:F131"/>
+    <mergeCell ref="E108:G108"/>
+    <mergeCell ref="E95:G95"/>
+    <mergeCell ref="E89:G89"/>
+    <mergeCell ref="E104:G104"/>
+    <mergeCell ref="F80:G80"/>
+    <mergeCell ref="F70:G70"/>
+    <mergeCell ref="F79:G79"/>
+    <mergeCell ref="C21:G21"/>
+    <mergeCell ref="F72:G72"/>
+    <mergeCell ref="F81:G81"/>
+    <mergeCell ref="C23:G23"/>
+    <mergeCell ref="F56:G56"/>
+    <mergeCell ref="F71:G71"/>
+    <mergeCell ref="E106:G106"/>
+    <mergeCell ref="B143:F143"/>
+    <mergeCell ref="B133:F133"/>
+    <mergeCell ref="B142:F142"/>
+    <mergeCell ref="E92:G92"/>
+    <mergeCell ref="F57:G57"/>
+    <mergeCell ref="C18:G18"/>
+    <mergeCell ref="E107:G107"/>
+    <mergeCell ref="B135:F135"/>
+    <mergeCell ref="B144:F144"/>
+    <mergeCell ref="B125:F125"/>
+    <mergeCell ref="F63:G63"/>
+    <mergeCell ref="B134:F134"/>
+    <mergeCell ref="E114:G114"/>
+    <mergeCell ref="F74:G74"/>
+    <mergeCell ref="E86:G86"/>
+    <mergeCell ref="C20:G20"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="D35:G35"/>
+    <mergeCell ref="E94:G94"/>
+    <mergeCell ref="F76:G76"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="D34:G34"/>
+    <mergeCell ref="C22:G22"/>
+    <mergeCell ref="F66:G66"/>
+    <mergeCell ref="B148:F148"/>
+    <mergeCell ref="F75:G75"/>
+    <mergeCell ref="A119:G119"/>
+    <mergeCell ref="C12:G12"/>
+    <mergeCell ref="F62:G62"/>
+    <mergeCell ref="E112:G112"/>
+    <mergeCell ref="D36:G36"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="F61:G61"/>
+    <mergeCell ref="E111:G111"/>
+    <mergeCell ref="E98:G98"/>
+    <mergeCell ref="B124:F124"/>
+    <mergeCell ref="E88:G88"/>
+    <mergeCell ref="F64:G64"/>
+    <mergeCell ref="A5:G5"/>
+    <mergeCell ref="B126:F126"/>
+    <mergeCell ref="F73:G73"/>
+    <mergeCell ref="C24:G24"/>
+    <mergeCell ref="B141:F141"/>
+    <mergeCell ref="B150:F150"/>
+    <mergeCell ref="C26:G26"/>
+    <mergeCell ref="B152:F152"/>
+    <mergeCell ref="C10:G10"/>
+    <mergeCell ref="C16:G16"/>
+    <mergeCell ref="E116:G116"/>
+    <mergeCell ref="C25:G25"/>
+    <mergeCell ref="B136:F136"/>
+    <mergeCell ref="E113:G113"/>
+    <mergeCell ref="B145:F145"/>
+    <mergeCell ref="A82:G82"/>
+    <mergeCell ref="E100:G100"/>
+    <mergeCell ref="E115:G115"/>
+    <mergeCell ref="A6:G6"/>
+    <mergeCell ref="E102:G102"/>
+    <mergeCell ref="C11:G11"/>
+    <mergeCell ref="B128:F128"/>
+    <mergeCell ref="B137:F137"/>
+    <mergeCell ref="F77:G77"/>
+    <mergeCell ref="B139:F139"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="B123:F123"/>
+    <mergeCell ref="B154:F154"/>
+    <mergeCell ref="C13:G13"/>
+    <mergeCell ref="E87:G87"/>
+    <mergeCell ref="B138:F138"/>
+    <mergeCell ref="F78:G78"/>
+    <mergeCell ref="C15:G15"/>
+    <mergeCell ref="F65:G65"/>
+    <mergeCell ref="B140:F140"/>
+    <mergeCell ref="B155:F155"/>
+    <mergeCell ref="B149:F149"/>
+    <mergeCell ref="E90:G90"/>
+    <mergeCell ref="E105:G105"/>
+    <mergeCell ref="E99:G99"/>
+    <mergeCell ref="F59:G59"/>
+    <mergeCell ref="F55:G55"/>
+    <mergeCell ref="B151:F151"/>
+    <mergeCell ref="E101:G101"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="B132:F132"/>
+    <mergeCell ref="E91:G91"/>
+    <mergeCell ref="E85:G85"/>
+    <mergeCell ref="E93:G93"/>
+    <mergeCell ref="A7:G7"/>
+    <mergeCell ref="F58:G58"/>
+    <mergeCell ref="B127:F127"/>
+    <mergeCell ref="C17:G17"/>
+    <mergeCell ref="F67:G67"/>
+    <mergeCell ref="E117:G117"/>
+    <mergeCell ref="F60:G60"/>
+    <mergeCell ref="C19:G19"/>
+    <mergeCell ref="B153:F153"/>
+    <mergeCell ref="E103:G103"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F30"/>
@@ -1327,7 +4610,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="12" t="inlineStr">
         <is>
@@ -1670,7 +4952,6 @@
         <v/>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="15.75" customHeight="1">
       <c r="A18" s="12" t="inlineStr">
         <is>
@@ -2014,13 +5295,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.542857142857139" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -2123,7 +5404,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>LIS trả chỉ số thiếu mã và tên chỉ số, gần như toàn bộ ở Tổng phân tích tế bào máu 22.0121.1369</t>
+          <t>LIS trả chỉ số thiếu mã và tên chỉ số, 91% ở Tổng phân tích tế bào máu 22.0121.1369 (còn lại: đường máu mao mạch 01.0281.1510, khí máu 23.0103.1531)</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -2243,7 +5524,7 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Danh mục DVKT cơ sở 01929 thiếu (8.123 dòng so với 15.660 của 37470), nhiều mã CĐHA (X-quang ngực 18.0119.0028); tên DVKT khác tên phê duyệt</t>
+          <t>Danh mục DVKT cơ sở 01929 thiếu (8.595 dòng so với 15.723 của 37470), nhiều mã CĐHA (X-quang ngực 18.0119.0028); tên DVKT khác tên phê duyệt</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
@@ -2423,12 +5704,12 @@
       </c>
       <c r="D16" s="6" t="inlineStr">
         <is>
-          <t>Bác sĩ chỉ định = người thực hiện; tóm tắt kết quả ghi "xem hs BA"; diễn biến sao chép; mã bệnh Z00; liều dùng sai định dạng; thiếu PP điều trị</t>
+          <t>Bác sĩ chỉ định = người thực hiện; tóm tắt kết quả ghi "xem hs BA"; diễn biến sao chép; liều dùng sai định dạng; thiếu PP điều trị</t>
         </is>
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Cùng BS 4.779; tóm tắt ngắn 7.258; Z00 2; diễn biến trùng 1.583 HS</t>
+          <t>Cùng BS 4.779; tóm tắt ngắn 7.258; diễn biến trùng 1.583 HS</t>
         </is>
       </c>
       <c r="F16" s="6" t="inlineStr">
@@ -2453,12 +5734,12 @@
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>Thiếu CCCD, dân tộc, nghề nghiệp; mã nơi đi/đến gõ sai</t>
+          <t>Thiếu CCCD, dân tộc; mã nơi đi/đến gõ sai</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>CCCD 420; nghề nghiệp 0 HS</t>
+          <t>CCCD 420 HS</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -2497,13 +5778,14 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="1" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2818,13 +6100,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P260"/>
+  <dimension ref="A1:P223"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.542857142857139" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18347,43 +21629,6 @@
       </c>
     </row>
     <row r="223"/>
-    <row r="224"/>
-    <row r="225"/>
-    <row r="226"/>
-    <row r="227"/>
-    <row r="228"/>
-    <row r="229"/>
-    <row r="230"/>
-    <row r="231"/>
-    <row r="232"/>
-    <row r="233"/>
-    <row r="234"/>
-    <row r="235"/>
-    <row r="236"/>
-    <row r="237"/>
-    <row r="238"/>
-    <row r="239"/>
-    <row r="240"/>
-    <row r="241"/>
-    <row r="242"/>
-    <row r="243"/>
-    <row r="244"/>
-    <row r="245"/>
-    <row r="246"/>
-    <row r="247"/>
-    <row r="248"/>
-    <row r="249"/>
-    <row r="250"/>
-    <row r="251"/>
-    <row r="252"/>
-    <row r="253"/>
-    <row r="254"/>
-    <row r="255"/>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
-    <row r="260"/>
   </sheetData>
   <autoFilter ref="A4:P222"/>
   <conditionalFormatting sqref="E5:E222">
@@ -18414,7 +21659,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21288,7 +24533,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -21317,7 +24562,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>• Không dùng bảng lỗi đã ghi: bảng đó chứa kết quả của nhiều phiên bản quy tắc khác nhau. Kiểm lại toàn bộ cho số liệu đồng nhất theo quy tắc hiện hành; hồ sơ đã sửa và nạp lại được kiểm theo dữ liệu mới nhất.</t>
+          <t>• Đối chiếu: kết quả chạy lại khớp kết quả hệ thống đã ghi khi nạp (157.141 so với 157.205 cặp hồ sơ–mã lỗi; chênh lệch nhỏ do vài hồ sơ kiểm trước khi bản cập nhật quy tắc mới nhất có hiệu lực). Số trong tệp vì vậy cũng là số các đơn vị đang thấy trên màn hình Tiền giám định.</t>
         </is>
       </c>
     </row>

</xml_diff>